<commit_message>
Fix Chartres DS to only have concepts for th252
</commit_message>
<xml_diff>
--- a/src/main/resources/datasets/Import_Chartres_Projet.xlsx
+++ b/src/main/resources/datasets/Import_Chartres_Projet.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="252">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="251">
   <si>
     <t>Nom</t>
   </si>
@@ -189,10 +189,10 @@
       <rPr>
         <u val="single"/>
         <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Calibri"/>
+        <color indexed="11"/>
+        <rFont val="Arial"/>
       </rPr>
-      <t>https://thesaurus.mom.fr/?idc=4287983&amp;idt=th240</t>
+      <t>https://thesaurus.mom.fr/?idc=4290862&amp;idt=th252</t>
     </r>
   </si>
   <si>
@@ -264,10 +264,10 @@
       <rPr>
         <u val="single"/>
         <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Calibri"/>
+        <color indexed="11"/>
+        <rFont val="Arial"/>
       </rPr>
-      <t>https://thesaurus.mom.fr/?idc=4287984&amp;idt=th240</t>
+      <t>https://thesaurus.mom.fr/?idc=4290863&amp;idt=th252</t>
     </r>
   </si>
   <si>
@@ -293,10 +293,10 @@
       <rPr>
         <u val="single"/>
         <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Calibri"/>
+        <color indexed="11"/>
+        <rFont val="Arial"/>
       </rPr>
-      <t>https://thesaurus.mom.fr/?idc=4287985&amp;idt=th240</t>
+      <t>https://thesaurus.mom.fr/?idc=4290864&amp;idt=th252</t>
     </r>
   </si>
   <si>
@@ -339,10 +339,10 @@
       <rPr>
         <u val="single"/>
         <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Calibri"/>
+        <color indexed="11"/>
+        <rFont val="Arial"/>
       </rPr>
-      <t>https://thesaurus.mom.fr/?idc=4287540&amp;idt=th240</t>
+      <t>https://thesaurus.mom.fr/?idc=4286197&amp;idt=th252</t>
     </r>
   </si>
   <si>
@@ -445,17 +445,6 @@
     <t>Cuve carrée en briques rouges maçonnées sur deux rangs;</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <u val="single"/>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t>https://thesaurus.mom.fr/?idc=4287754&amp;idt=th240</t>
-    </r>
-  </si>
-  <si>
     <t>1024</t>
   </si>
   <si>
@@ -514,10 +503,10 @@
       <rPr>
         <u val="single"/>
         <sz val="10"/>
-        <color indexed="8"/>
+        <color indexed="11"/>
         <rFont val="Calibri"/>
       </rPr>
-      <t>https://thesaurus.mom.fr/?idc=4287988&amp;idt=th240</t>
+      <t>https://thesaurus.mom.fr/?idc=4290865&amp;idt=th252</t>
     </r>
   </si>
   <si>
@@ -998,7 +987,7 @@
     <numFmt numFmtId="0" formatCode="General"/>
     <numFmt numFmtId="59" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <sz val="10"/>
       <color indexed="8"/>
@@ -1024,6 +1013,12 @@
       <u val="single"/>
       <sz val="10"/>
       <color indexed="8"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <u val="single"/>
+      <sz val="10"/>
+      <color indexed="11"/>
       <name val="Calibri"/>
     </font>
     <font>
@@ -1675,13 +1670,13 @@
     <xf numFmtId="49" fontId="3" fillId="2" borderId="9" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="3" borderId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="6" fillId="3" borderId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="10" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="6" fillId="2" borderId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="7" fillId="2" borderId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="11" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
@@ -1699,28 +1694,28 @@
     <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="2" borderId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top"/>
-    </xf>
     <xf numFmtId="49" fontId="8" fillId="2" borderId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="8" fillId="2" borderId="14" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="9" fillId="2" borderId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="8" fillId="2" borderId="15" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="9" fillId="2" borderId="14" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="2" borderId="15" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="9" fillId="4" borderId="16" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="10" fillId="4" borderId="16" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="16" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="16" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="9" fillId="5" borderId="17" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="10" fillId="5" borderId="17" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="18" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
@@ -1729,7 +1724,7 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="19" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="9" fillId="5" borderId="20" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="10" fillId="5" borderId="20" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="21" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
@@ -1738,13 +1733,13 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="22" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="10" fillId="2" borderId="21" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="11" fillId="2" borderId="21" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="22" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="9" fillId="5" borderId="23" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="10" fillId="5" borderId="23" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="24" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
@@ -1759,13 +1754,13 @@
     <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="11" fillId="2" borderId="26" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="12" fillId="2" borderId="26" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="11" fillId="2" borderId="27" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="12" fillId="2" borderId="27" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="11" fillId="2" borderId="28" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="12" fillId="2" borderId="28" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="29" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
@@ -1801,10 +1796,10 @@
     <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="11" fillId="2" borderId="37" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="12" fillId="2" borderId="37" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="11" fillId="2" borderId="16" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="12" fillId="2" borderId="16" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="38" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
@@ -4146,7 +4141,7 @@
       </c>
       <c r="E25" s="13"/>
       <c r="F25" t="s" s="14">
-        <v>105</v>
+        <v>79</v>
       </c>
       <c r="G25" t="s" s="5">
         <v>46</v>
@@ -4171,10 +4166,10 @@
     </row>
     <row r="26" ht="13.75" customHeight="1">
       <c r="A26" t="s" s="2">
+        <v>105</v>
+      </c>
+      <c r="B26" t="s" s="2">
         <v>106</v>
-      </c>
-      <c r="B26" t="s" s="2">
-        <v>107</v>
       </c>
       <c r="C26" t="s" s="12">
         <v>43</v>
@@ -4209,10 +4204,10 @@
     </row>
     <row r="27" ht="13.75" customHeight="1">
       <c r="A27" t="s" s="2">
+        <v>107</v>
+      </c>
+      <c r="B27" t="s" s="2">
         <v>108</v>
-      </c>
-      <c r="B27" t="s" s="2">
-        <v>109</v>
       </c>
       <c r="C27" t="s" s="12">
         <v>43</v>
@@ -4247,10 +4242,10 @@
     </row>
     <row r="28" ht="13.75" customHeight="1">
       <c r="A28" t="s" s="2">
+        <v>109</v>
+      </c>
+      <c r="B28" t="s" s="2">
         <v>110</v>
-      </c>
-      <c r="B28" t="s" s="2">
-        <v>111</v>
       </c>
       <c r="C28" t="s" s="12">
         <v>43</v>
@@ -4285,10 +4280,10 @@
     </row>
     <row r="29" ht="13.75" customHeight="1">
       <c r="A29" t="s" s="2">
+        <v>111</v>
+      </c>
+      <c r="B29" t="s" s="2">
         <v>112</v>
-      </c>
-      <c r="B29" t="s" s="2">
-        <v>113</v>
       </c>
       <c r="C29" t="s" s="12">
         <v>43</v>
@@ -4323,10 +4318,10 @@
     </row>
     <row r="30" ht="13.75" customHeight="1">
       <c r="A30" t="s" s="2">
+        <v>113</v>
+      </c>
+      <c r="B30" t="s" s="2">
         <v>114</v>
-      </c>
-      <c r="B30" t="s" s="2">
-        <v>115</v>
       </c>
       <c r="C30" t="s" s="12">
         <v>43</v>
@@ -4361,10 +4356,10 @@
     </row>
     <row r="31" ht="13.75" customHeight="1">
       <c r="A31" t="s" s="2">
+        <v>115</v>
+      </c>
+      <c r="B31" t="s" s="2">
         <v>116</v>
-      </c>
-      <c r="B31" t="s" s="2">
-        <v>117</v>
       </c>
       <c r="C31" t="s" s="12">
         <v>43</v>
@@ -4399,10 +4394,10 @@
     </row>
     <row r="32" ht="13.75" customHeight="1">
       <c r="A32" t="s" s="2">
+        <v>117</v>
+      </c>
+      <c r="B32" t="s" s="2">
         <v>118</v>
-      </c>
-      <c r="B32" t="s" s="2">
-        <v>119</v>
       </c>
       <c r="C32" t="s" s="12">
         <v>43</v>
@@ -4437,10 +4432,10 @@
     </row>
     <row r="33" ht="13.75" customHeight="1">
       <c r="A33" t="s" s="2">
+        <v>119</v>
+      </c>
+      <c r="B33" t="s" s="2">
         <v>120</v>
-      </c>
-      <c r="B33" t="s" s="2">
-        <v>121</v>
       </c>
       <c r="C33" t="s" s="12">
         <v>43</v>
@@ -4450,7 +4445,7 @@
       </c>
       <c r="E33" s="13"/>
       <c r="F33" t="s" s="14">
-        <v>105</v>
+        <v>79</v>
       </c>
       <c r="G33" t="s" s="5">
         <v>46</v>
@@ -4475,10 +4470,10 @@
     </row>
     <row r="34" ht="13.75" customHeight="1">
       <c r="A34" t="s" s="2">
+        <v>121</v>
+      </c>
+      <c r="B34" t="s" s="2">
         <v>122</v>
-      </c>
-      <c r="B34" t="s" s="2">
-        <v>123</v>
       </c>
       <c r="C34" t="s" s="12">
         <v>43</v>
@@ -4488,7 +4483,7 @@
       </c>
       <c r="E34" s="13"/>
       <c r="F34" t="s" s="14">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="G34" t="s" s="5">
         <v>46</v>
@@ -4513,10 +4508,10 @@
     </row>
     <row r="35" ht="13.75" customHeight="1">
       <c r="A35" t="s" s="2">
+        <v>124</v>
+      </c>
+      <c r="B35" t="s" s="2">
         <v>125</v>
-      </c>
-      <c r="B35" t="s" s="2">
-        <v>126</v>
       </c>
       <c r="C35" t="s" s="12">
         <v>43</v>
@@ -4551,10 +4546,10 @@
     </row>
     <row r="36" ht="13.75" customHeight="1">
       <c r="A36" t="s" s="2">
+        <v>126</v>
+      </c>
+      <c r="B36" t="s" s="2">
         <v>127</v>
-      </c>
-      <c r="B36" t="s" s="2">
-        <v>128</v>
       </c>
       <c r="C36" t="s" s="12">
         <v>43</v>
@@ -4564,7 +4559,7 @@
       </c>
       <c r="E36" s="13"/>
       <c r="F36" t="s" s="14">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="G36" t="s" s="5">
         <v>46</v>
@@ -4589,10 +4584,10 @@
     </row>
     <row r="37" ht="13.75" customHeight="1">
       <c r="A37" t="s" s="2">
+        <v>128</v>
+      </c>
+      <c r="B37" t="s" s="2">
         <v>129</v>
-      </c>
-      <c r="B37" t="s" s="2">
-        <v>130</v>
       </c>
       <c r="C37" t="s" s="12">
         <v>43</v>
@@ -4627,10 +4622,10 @@
     </row>
     <row r="38" ht="13.75" customHeight="1">
       <c r="A38" t="s" s="2">
+        <v>130</v>
+      </c>
+      <c r="B38" t="s" s="2">
         <v>131</v>
-      </c>
-      <c r="B38" t="s" s="2">
-        <v>132</v>
       </c>
       <c r="C38" t="s" s="12">
         <v>43</v>
@@ -4665,10 +4660,10 @@
     </row>
     <row r="39" ht="13.75" customHeight="1">
       <c r="A39" t="s" s="2">
+        <v>132</v>
+      </c>
+      <c r="B39" t="s" s="2">
         <v>133</v>
-      </c>
-      <c r="B39" t="s" s="2">
-        <v>134</v>
       </c>
       <c r="C39" t="s" s="12">
         <v>43</v>
@@ -4678,7 +4673,7 @@
       </c>
       <c r="E39" s="13"/>
       <c r="F39" t="s" s="14">
-        <v>105</v>
+        <v>123</v>
       </c>
       <c r="G39" t="s" s="5">
         <v>46</v>
@@ -4703,10 +4698,10 @@
     </row>
     <row r="40" ht="13.75" customHeight="1">
       <c r="A40" t="s" s="2">
+        <v>134</v>
+      </c>
+      <c r="B40" t="s" s="2">
         <v>135</v>
-      </c>
-      <c r="B40" t="s" s="2">
-        <v>136</v>
       </c>
       <c r="C40" t="s" s="12">
         <v>43</v>
@@ -4741,10 +4736,10 @@
     </row>
     <row r="41" ht="13.75" customHeight="1">
       <c r="A41" t="s" s="2">
+        <v>136</v>
+      </c>
+      <c r="B41" t="s" s="2">
         <v>137</v>
-      </c>
-      <c r="B41" t="s" s="2">
-        <v>138</v>
       </c>
       <c r="C41" t="s" s="12">
         <v>43</v>
@@ -4779,10 +4774,10 @@
     </row>
     <row r="42" ht="13.75" customHeight="1">
       <c r="A42" t="s" s="2">
+        <v>138</v>
+      </c>
+      <c r="B42" t="s" s="2">
         <v>139</v>
-      </c>
-      <c r="B42" t="s" s="2">
-        <v>140</v>
       </c>
       <c r="C42" t="s" s="12">
         <v>43</v>
@@ -4817,10 +4812,10 @@
     </row>
     <row r="43" ht="13.75" customHeight="1">
       <c r="A43" t="s" s="2">
+        <v>140</v>
+      </c>
+      <c r="B43" t="s" s="2">
         <v>141</v>
-      </c>
-      <c r="B43" t="s" s="2">
-        <v>142</v>
       </c>
       <c r="C43" t="s" s="12">
         <v>43</v>
@@ -4855,10 +4850,10 @@
     </row>
     <row r="44" ht="13.75" customHeight="1">
       <c r="A44" t="s" s="2">
+        <v>142</v>
+      </c>
+      <c r="B44" t="s" s="2">
         <v>143</v>
-      </c>
-      <c r="B44" t="s" s="2">
-        <v>144</v>
       </c>
       <c r="C44" t="s" s="12">
         <v>43</v>
@@ -4893,10 +4888,10 @@
     </row>
     <row r="45" ht="13.75" customHeight="1">
       <c r="A45" t="s" s="2">
+        <v>144</v>
+      </c>
+      <c r="B45" t="s" s="2">
         <v>145</v>
-      </c>
-      <c r="B45" t="s" s="2">
-        <v>146</v>
       </c>
       <c r="C45" t="s" s="12">
         <v>43</v>
@@ -4931,10 +4926,10 @@
     </row>
     <row r="46" ht="13.75" customHeight="1">
       <c r="A46" t="s" s="2">
+        <v>146</v>
+      </c>
+      <c r="B46" t="s" s="2">
         <v>147</v>
-      </c>
-      <c r="B46" t="s" s="2">
-        <v>148</v>
       </c>
       <c r="C46" t="s" s="12">
         <v>43</v>
@@ -4969,10 +4964,10 @@
     </row>
     <row r="47" ht="13.75" customHeight="1">
       <c r="A47" t="s" s="2">
+        <v>148</v>
+      </c>
+      <c r="B47" t="s" s="2">
         <v>149</v>
-      </c>
-      <c r="B47" t="s" s="2">
-        <v>150</v>
       </c>
       <c r="C47" t="s" s="12">
         <v>43</v>
@@ -5007,10 +5002,10 @@
     </row>
     <row r="48" ht="13.75" customHeight="1">
       <c r="A48" t="s" s="17">
+        <v>150</v>
+      </c>
+      <c r="B48" t="s" s="17">
         <v>151</v>
-      </c>
-      <c r="B48" t="s" s="17">
-        <v>152</v>
       </c>
       <c r="C48" t="s" s="18">
         <v>43</v>
@@ -5045,11 +5040,11 @@
     </row>
     <row r="49" ht="14.7" customHeight="1">
       <c r="A49" t="s" s="19">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B49" s="20"/>
       <c r="C49" t="s" s="21">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D49" s="22"/>
       <c r="E49" s="6"/>
@@ -5073,11 +5068,11 @@
     </row>
     <row r="50" ht="14.7" customHeight="1">
       <c r="A50" t="s" s="19">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B50" s="20"/>
       <c r="C50" t="s" s="21">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D50" s="22"/>
       <c r="E50" s="6"/>
@@ -5101,11 +5096,11 @@
     </row>
     <row r="51" ht="14.7" customHeight="1">
       <c r="A51" t="s" s="19">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B51" s="20"/>
       <c r="C51" t="s" s="21">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D51" s="22"/>
       <c r="E51" s="6"/>
@@ -5129,11 +5124,11 @@
     </row>
     <row r="52" ht="14.7" customHeight="1">
       <c r="A52" t="s" s="19">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B52" s="20"/>
       <c r="C52" t="s" s="21">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D52" s="22"/>
       <c r="E52" s="6"/>
@@ -5157,11 +5152,11 @@
     </row>
     <row r="53" ht="14.7" customHeight="1">
       <c r="A53" t="s" s="19">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B53" s="20"/>
       <c r="C53" t="s" s="21">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D53" s="22"/>
       <c r="E53" s="6"/>
@@ -5185,11 +5180,11 @@
     </row>
     <row r="54" ht="14.7" customHeight="1">
       <c r="A54" t="s" s="19">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B54" s="20"/>
       <c r="C54" t="s" s="21">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D54" s="22"/>
       <c r="E54" s="6"/>
@@ -5213,11 +5208,11 @@
     </row>
     <row r="55" ht="14.7" customHeight="1">
       <c r="A55" t="s" s="19">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B55" s="20"/>
       <c r="C55" t="s" s="21">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D55" s="22"/>
       <c r="E55" s="6"/>
@@ -5241,11 +5236,11 @@
     </row>
     <row r="56" ht="14.7" customHeight="1">
       <c r="A56" t="s" s="19">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B56" s="20"/>
       <c r="C56" t="s" s="21">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D56" s="22"/>
       <c r="E56" s="6"/>
@@ -5269,11 +5264,11 @@
     </row>
     <row r="57" ht="14.7" customHeight="1">
       <c r="A57" t="s" s="19">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B57" s="20"/>
       <c r="C57" t="s" s="21">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D57" s="22"/>
       <c r="E57" s="6"/>
@@ -5297,11 +5292,11 @@
     </row>
     <row r="58" ht="14.7" customHeight="1">
       <c r="A58" t="s" s="19">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B58" s="20"/>
       <c r="C58" t="s" s="21">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D58" s="22"/>
       <c r="E58" s="6"/>
@@ -5325,11 +5320,11 @@
     </row>
     <row r="59" ht="13.65" customHeight="1">
       <c r="A59" t="s" s="19">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B59" s="20"/>
       <c r="C59" t="s" s="21">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D59" s="22"/>
       <c r="E59" s="6"/>
@@ -5353,11 +5348,11 @@
     </row>
     <row r="60" ht="13.65" customHeight="1">
       <c r="A60" t="s" s="19">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B60" s="20"/>
       <c r="C60" t="s" s="21">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D60" s="22"/>
       <c r="E60" s="6"/>
@@ -5381,11 +5376,11 @@
     </row>
     <row r="61" ht="13.65" customHeight="1">
       <c r="A61" t="s" s="24">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B61" s="25"/>
       <c r="C61" t="s" s="24">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D61" s="6"/>
       <c r="E61" s="6"/>
@@ -5409,11 +5404,11 @@
     </row>
     <row r="62" ht="13.65" customHeight="1">
       <c r="A62" t="s" s="2">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B62" s="6"/>
       <c r="C62" t="s" s="2">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D62" s="6"/>
       <c r="E62" s="6"/>
@@ -5437,11 +5432,11 @@
     </row>
     <row r="63" ht="13.65" customHeight="1">
       <c r="A63" t="s" s="2">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B63" s="6"/>
       <c r="C63" t="s" s="2">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D63" s="6"/>
       <c r="E63" s="6"/>
@@ -5465,11 +5460,11 @@
     </row>
     <row r="64" ht="13.65" customHeight="1">
       <c r="A64" t="s" s="2">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B64" s="6"/>
       <c r="C64" t="s" s="2">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D64" s="6"/>
       <c r="E64" s="6"/>
@@ -5493,11 +5488,11 @@
     </row>
     <row r="65" ht="13.65" customHeight="1">
       <c r="A65" t="s" s="2">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B65" s="6"/>
       <c r="C65" t="s" s="2">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D65" s="6"/>
       <c r="E65" s="6"/>
@@ -5521,11 +5516,11 @@
     </row>
     <row r="66" ht="13.65" customHeight="1">
       <c r="A66" t="s" s="2">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B66" s="6"/>
       <c r="C66" t="s" s="2">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D66" s="6"/>
       <c r="E66" s="6"/>
@@ -5549,11 +5544,11 @@
     </row>
     <row r="67" ht="13.65" customHeight="1">
       <c r="A67" t="s" s="2">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B67" s="6"/>
       <c r="C67" t="s" s="2">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D67" s="6"/>
       <c r="E67" s="6"/>
@@ -5577,11 +5572,11 @@
     </row>
     <row r="68" ht="13.65" customHeight="1">
       <c r="A68" t="s" s="2">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B68" s="6"/>
       <c r="C68" t="s" s="2">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D68" s="6"/>
       <c r="E68" s="6"/>
@@ -5605,11 +5600,11 @@
     </row>
     <row r="69" ht="13.65" customHeight="1">
       <c r="A69" t="s" s="2">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B69" s="6"/>
       <c r="C69" t="s" s="2">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D69" s="6"/>
       <c r="E69" s="6"/>
@@ -5633,11 +5628,11 @@
     </row>
     <row r="70" ht="13.65" customHeight="1">
       <c r="A70" t="s" s="2">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B70" s="6"/>
       <c r="C70" t="s" s="2">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D70" s="6"/>
       <c r="E70" s="6"/>
@@ -5661,11 +5656,11 @@
     </row>
     <row r="71" ht="13.65" customHeight="1">
       <c r="A71" t="s" s="2">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B71" s="6"/>
       <c r="C71" t="s" s="2">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D71" s="6"/>
       <c r="E71" s="6"/>
@@ -5689,11 +5684,11 @@
     </row>
     <row r="72" ht="13.65" customHeight="1">
       <c r="A72" t="s" s="2">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B72" s="6"/>
       <c r="C72" t="s" s="2">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D72" s="6"/>
       <c r="E72" s="6"/>
@@ -5717,11 +5712,11 @@
     </row>
     <row r="73" ht="13.65" customHeight="1">
       <c r="A73" t="s" s="2">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B73" s="6"/>
       <c r="C73" t="s" s="2">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D73" s="6"/>
       <c r="E73" s="6"/>
@@ -5745,11 +5740,11 @@
     </row>
     <row r="74" ht="13.65" customHeight="1">
       <c r="A74" t="s" s="2">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B74" s="6"/>
       <c r="C74" t="s" s="2">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="D74" s="6"/>
       <c r="E74" s="6"/>
@@ -5773,11 +5768,11 @@
     </row>
     <row r="75" ht="13.65" customHeight="1">
       <c r="A75" t="s" s="2">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B75" s="6"/>
       <c r="C75" t="s" s="2">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="D75" s="6"/>
       <c r="E75" s="6"/>
@@ -5801,11 +5796,11 @@
     </row>
     <row r="76" ht="13.65" customHeight="1">
       <c r="A76" t="s" s="2">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B76" s="6"/>
       <c r="C76" t="s" s="2">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="D76" s="6"/>
       <c r="E76" s="6"/>
@@ -5829,11 +5824,11 @@
     </row>
     <row r="77" ht="13.65" customHeight="1">
       <c r="A77" t="s" s="2">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B77" s="6"/>
       <c r="C77" t="s" s="2">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="D77" s="6"/>
       <c r="E77" s="6"/>
@@ -5857,11 +5852,11 @@
     </row>
     <row r="78" ht="13.65" customHeight="1">
       <c r="A78" t="s" s="2">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B78" s="6"/>
       <c r="C78" t="s" s="2">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="D78" s="6"/>
       <c r="E78" s="6"/>
@@ -5885,11 +5880,11 @@
     </row>
     <row r="79" ht="13.65" customHeight="1">
       <c r="A79" t="s" s="2">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B79" s="6"/>
       <c r="C79" t="s" s="2">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="D79" s="6"/>
       <c r="E79" s="6"/>
@@ -5913,11 +5908,11 @@
     </row>
     <row r="80" ht="13.65" customHeight="1">
       <c r="A80" t="s" s="2">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B80" s="6"/>
       <c r="C80" t="s" s="2">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="D80" s="6"/>
       <c r="E80" s="6"/>
@@ -20631,13 +20626,13 @@
   <hyperlinks>
     <hyperlink ref="C2" r:id="rId1" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287627&amp;idt=th252"/>
     <hyperlink ref="D2" r:id="rId2" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287638&amp;idt=th252"/>
-    <hyperlink ref="F2" r:id="rId3" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287983&amp;idt=th240"/>
+    <hyperlink ref="F2" r:id="rId3" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4290862&amp;idt=th252"/>
     <hyperlink ref="C3" r:id="rId4" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287627&amp;idt=th252"/>
     <hyperlink ref="D3" r:id="rId5" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287638&amp;idt=th252"/>
-    <hyperlink ref="F3" r:id="rId6" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287983&amp;idt=th240"/>
+    <hyperlink ref="F3" r:id="rId6" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4290862&amp;idt=th252"/>
     <hyperlink ref="C4" r:id="rId7" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287627&amp;idt=th252"/>
     <hyperlink ref="D4" r:id="rId8" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287638&amp;idt=th252"/>
-    <hyperlink ref="F4" r:id="rId9" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287983&amp;idt=th240"/>
+    <hyperlink ref="F4" r:id="rId9" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4290862&amp;idt=th252"/>
     <hyperlink ref="C5" r:id="rId10" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287627&amp;idt=th252"/>
     <hyperlink ref="D5" r:id="rId11" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287638&amp;idt=th252"/>
     <hyperlink ref="F5" r:id="rId12" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287744&amp;idt=th252"/>
@@ -20646,37 +20641,37 @@
     <hyperlink ref="F6" r:id="rId15" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287682&amp;idt=th252"/>
     <hyperlink ref="C7" r:id="rId16" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287627&amp;idt=th252"/>
     <hyperlink ref="D7" r:id="rId17" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287638&amp;idt=th252"/>
-    <hyperlink ref="F7" r:id="rId18" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287984&amp;idt=th240"/>
+    <hyperlink ref="F7" r:id="rId18" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4290863&amp;idt=th252"/>
     <hyperlink ref="C8" r:id="rId19" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287627&amp;idt=th252"/>
     <hyperlink ref="D8" r:id="rId20" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287638&amp;idt=th252"/>
-    <hyperlink ref="F8" r:id="rId21" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287984&amp;idt=th240"/>
+    <hyperlink ref="F8" r:id="rId21" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4290863&amp;idt=th252"/>
     <hyperlink ref="C9" r:id="rId22" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287627&amp;idt=th252"/>
     <hyperlink ref="D9" r:id="rId23" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287638&amp;idt=th252"/>
     <hyperlink ref="F9" r:id="rId24" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287682&amp;idt=th252"/>
     <hyperlink ref="C10" r:id="rId25" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287627&amp;idt=th252"/>
     <hyperlink ref="D10" r:id="rId26" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287638&amp;idt=th252"/>
-    <hyperlink ref="F10" r:id="rId27" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287985&amp;idt=th240"/>
+    <hyperlink ref="F10" r:id="rId27" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4290864&amp;idt=th252"/>
     <hyperlink ref="C11" r:id="rId28" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287627&amp;idt=th252"/>
     <hyperlink ref="D11" r:id="rId29" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287638&amp;idt=th252"/>
     <hyperlink ref="F11" r:id="rId30" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287682&amp;idt=th252"/>
     <hyperlink ref="C12" r:id="rId31" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287627&amp;idt=th252"/>
     <hyperlink ref="D12" r:id="rId32" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287638&amp;idt=th252"/>
-    <hyperlink ref="F12" r:id="rId33" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287983&amp;idt=th240"/>
+    <hyperlink ref="F12" r:id="rId33" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4290862&amp;idt=th252"/>
     <hyperlink ref="C13" r:id="rId34" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287627&amp;idt=th252"/>
     <hyperlink ref="D13" r:id="rId35" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287638&amp;idt=th252"/>
     <hyperlink ref="F13" r:id="rId36" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287682&amp;idt=th252"/>
     <hyperlink ref="C14" r:id="rId37" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287627&amp;idt=th252"/>
     <hyperlink ref="D14" r:id="rId38" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287639&amp;idt=th252"/>
-    <hyperlink ref="F14" r:id="rId39" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287540&amp;idt=th240"/>
+    <hyperlink ref="F14" r:id="rId39" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4286197&amp;idt=th252"/>
     <hyperlink ref="C15" r:id="rId40" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287627&amp;idt=th252"/>
     <hyperlink ref="D15" r:id="rId41" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287638&amp;idt=th252"/>
     <hyperlink ref="F15" r:id="rId42" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287680&amp;idt=th252"/>
     <hyperlink ref="C16" r:id="rId43" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287627&amp;idt=th252"/>
     <hyperlink ref="D16" r:id="rId44" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287639&amp;idt=th252"/>
-    <hyperlink ref="F16" r:id="rId45" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287540&amp;idt=th240"/>
+    <hyperlink ref="F16" r:id="rId45" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4286197&amp;idt=th252"/>
     <hyperlink ref="C17" r:id="rId46" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287627&amp;idt=th252"/>
     <hyperlink ref="D17" r:id="rId47" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287639&amp;idt=th252"/>
-    <hyperlink ref="F17" r:id="rId48" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287540&amp;idt=th240"/>
+    <hyperlink ref="F17" r:id="rId48" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4286197&amp;idt=th252"/>
     <hyperlink ref="C18" r:id="rId49" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287627&amp;idt=th252"/>
     <hyperlink ref="D18" r:id="rId50" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287638&amp;idt=th252"/>
     <hyperlink ref="F18" r:id="rId51" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287744&amp;idt=th252"/>
@@ -20691,19 +20686,19 @@
     <hyperlink ref="F21" r:id="rId60" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287680&amp;idt=th252"/>
     <hyperlink ref="C22" r:id="rId61" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287627&amp;idt=th252"/>
     <hyperlink ref="D22" r:id="rId62" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287638&amp;idt=th252"/>
-    <hyperlink ref="F22" r:id="rId63" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287984&amp;idt=th240"/>
+    <hyperlink ref="F22" r:id="rId63" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4290863&amp;idt=th252"/>
     <hyperlink ref="C23" r:id="rId64" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287627&amp;idt=th252"/>
     <hyperlink ref="D23" r:id="rId65" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287638&amp;idt=th252"/>
     <hyperlink ref="F23" r:id="rId66" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287708&amp;idt=th252"/>
     <hyperlink ref="C24" r:id="rId67" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287627&amp;idt=th252"/>
     <hyperlink ref="D24" r:id="rId68" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287639&amp;idt=th252"/>
-    <hyperlink ref="F24" r:id="rId69" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287540&amp;idt=th240"/>
+    <hyperlink ref="F24" r:id="rId69" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4286197&amp;idt=th252"/>
     <hyperlink ref="C25" r:id="rId70" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287627&amp;idt=th252"/>
     <hyperlink ref="D25" r:id="rId71" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287638&amp;idt=th252"/>
-    <hyperlink ref="F25" r:id="rId72" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287754&amp;idt=th240"/>
+    <hyperlink ref="F25" r:id="rId72" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4286197&amp;idt=th252"/>
     <hyperlink ref="C26" r:id="rId73" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287627&amp;idt=th252"/>
     <hyperlink ref="D26" r:id="rId74" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287638&amp;idt=th252"/>
-    <hyperlink ref="F26" r:id="rId75" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287985&amp;idt=th240"/>
+    <hyperlink ref="F26" r:id="rId75" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4290864&amp;idt=th252"/>
     <hyperlink ref="C27" r:id="rId76" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287627&amp;idt=th252"/>
     <hyperlink ref="D27" r:id="rId77" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287638&amp;idt=th252"/>
     <hyperlink ref="F27" r:id="rId78" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287708&amp;idt=th252"/>
@@ -20712,7 +20707,7 @@
     <hyperlink ref="F28" r:id="rId81" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287744&amp;idt=th252"/>
     <hyperlink ref="C29" r:id="rId82" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287627&amp;idt=th252"/>
     <hyperlink ref="D29" r:id="rId83" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287639&amp;idt=th252"/>
-    <hyperlink ref="F29" r:id="rId84" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287540&amp;idt=th240"/>
+    <hyperlink ref="F29" r:id="rId84" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4286197&amp;idt=th252"/>
     <hyperlink ref="C30" r:id="rId85" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287627&amp;idt=th252"/>
     <hyperlink ref="D30" r:id="rId86" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287638&amp;idt=th252"/>
     <hyperlink ref="F30" r:id="rId87" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287708&amp;idt=th252"/>
@@ -20724,16 +20719,16 @@
     <hyperlink ref="F32" r:id="rId93" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287708&amp;idt=th252"/>
     <hyperlink ref="C33" r:id="rId94" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287627&amp;idt=th252"/>
     <hyperlink ref="D33" r:id="rId95" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287638&amp;idt=th252"/>
-    <hyperlink ref="F33" r:id="rId96" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287754&amp;idt=th240"/>
+    <hyperlink ref="F33" r:id="rId96" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4286197&amp;idt=th252"/>
     <hyperlink ref="C34" r:id="rId97" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287627&amp;idt=th252"/>
     <hyperlink ref="D34" r:id="rId98" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287638&amp;idt=th252"/>
-    <hyperlink ref="F34" r:id="rId99" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287988&amp;idt=th240"/>
+    <hyperlink ref="F34" r:id="rId99" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4290865&amp;idt=th252"/>
     <hyperlink ref="C35" r:id="rId100" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287627&amp;idt=th252"/>
     <hyperlink ref="D35" r:id="rId101" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287638&amp;idt=th252"/>
     <hyperlink ref="F35" r:id="rId102" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287708&amp;idt=th252"/>
     <hyperlink ref="C36" r:id="rId103" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287627&amp;idt=th252"/>
     <hyperlink ref="D36" r:id="rId104" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287638&amp;idt=th252"/>
-    <hyperlink ref="F36" r:id="rId105" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287988&amp;idt=th240"/>
+    <hyperlink ref="F36" r:id="rId105" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4290865&amp;idt=th252"/>
     <hyperlink ref="C37" r:id="rId106" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287627&amp;idt=th252"/>
     <hyperlink ref="D37" r:id="rId107" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287638&amp;idt=th252"/>
     <hyperlink ref="F37" r:id="rId108" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287708&amp;idt=th252"/>
@@ -20742,7 +20737,7 @@
     <hyperlink ref="F38" r:id="rId111" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287708&amp;idt=th252"/>
     <hyperlink ref="C39" r:id="rId112" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287627&amp;idt=th252"/>
     <hyperlink ref="D39" r:id="rId113" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287638&amp;idt=th252"/>
-    <hyperlink ref="F39" r:id="rId114" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287754&amp;idt=th240"/>
+    <hyperlink ref="F39" r:id="rId114" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4290865&amp;idt=th252"/>
     <hyperlink ref="C40" r:id="rId115" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287627&amp;idt=th252"/>
     <hyperlink ref="D40" r:id="rId116" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287638&amp;idt=th252"/>
     <hyperlink ref="F40" r:id="rId117" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287708&amp;idt=th252"/>
@@ -20757,7 +20752,7 @@
     <hyperlink ref="F43" r:id="rId126" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287682&amp;idt=th252"/>
     <hyperlink ref="C44" r:id="rId127" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287627&amp;idt=th252"/>
     <hyperlink ref="D44" r:id="rId128" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287638&amp;idt=th252"/>
-    <hyperlink ref="F44" r:id="rId129" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287984&amp;idt=th240"/>
+    <hyperlink ref="F44" r:id="rId129" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4290863&amp;idt=th252"/>
     <hyperlink ref="C45" r:id="rId130" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287627&amp;idt=th252"/>
     <hyperlink ref="D45" r:id="rId131" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287638&amp;idt=th252"/>
     <hyperlink ref="F45" r:id="rId132" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287708&amp;idt=th252"/>
@@ -20766,7 +20761,7 @@
     <hyperlink ref="F46" r:id="rId135" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287708&amp;idt=th252"/>
     <hyperlink ref="C47" r:id="rId136" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287627&amp;idt=th252"/>
     <hyperlink ref="D47" r:id="rId137" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287639&amp;idt=th252"/>
-    <hyperlink ref="F47" r:id="rId138" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287540&amp;idt=th240"/>
+    <hyperlink ref="F47" r:id="rId138" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4286197&amp;idt=th252"/>
     <hyperlink ref="C48" r:id="rId139" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287627&amp;idt=th252"/>
     <hyperlink ref="D48" r:id="rId140" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287638&amp;idt=th252"/>
     <hyperlink ref="F48" r:id="rId141" location="" tooltip="" display="https://thesaurus.mom.fr/?idc=4287680&amp;idt=th252"/>
@@ -20835,39 +20830,39 @@
         <v>27</v>
       </c>
       <c r="B1" t="s" s="17">
+        <v>187</v>
+      </c>
+      <c r="C1" t="s" s="17">
         <v>188</v>
       </c>
-      <c r="C1" t="s" s="17">
+      <c r="D1" t="s" s="17">
         <v>189</v>
-      </c>
-      <c r="D1" t="s" s="17">
-        <v>190</v>
       </c>
       <c r="E1" t="s" s="17">
         <v>34</v>
       </c>
       <c r="F1" t="s" s="2">
+        <v>190</v>
+      </c>
+      <c r="G1" t="s" s="2">
         <v>191</v>
       </c>
-      <c r="G1" t="s" s="2">
+      <c r="H1" t="s" s="17">
         <v>192</v>
-      </c>
-      <c r="H1" t="s" s="17">
-        <v>193</v>
       </c>
     </row>
     <row r="2" ht="14.7" customHeight="1">
       <c r="A2" t="s" s="19">
+        <v>193</v>
+      </c>
+      <c r="B2" t="s" s="27">
         <v>194</v>
       </c>
-      <c r="B2" t="s" s="27">
+      <c r="C2" t="s" s="28">
         <v>195</v>
       </c>
-      <c r="C2" t="s" s="28">
+      <c r="D2" t="s" s="27">
         <v>196</v>
-      </c>
-      <c r="D2" t="s" s="27">
-        <v>197</v>
       </c>
       <c r="E2" t="s" s="29">
         <v>6</v>
@@ -20884,16 +20879,16 @@
     </row>
     <row r="3" ht="14.7" customHeight="1">
       <c r="A3" t="s" s="19">
+        <v>197</v>
+      </c>
+      <c r="B3" t="s" s="27">
+        <v>194</v>
+      </c>
+      <c r="C3" t="s" s="27">
         <v>198</v>
       </c>
-      <c r="B3" t="s" s="27">
-        <v>195</v>
-      </c>
-      <c r="C3" t="s" s="27">
+      <c r="D3" t="s" s="27">
         <v>199</v>
-      </c>
-      <c r="D3" t="s" s="27">
-        <v>200</v>
       </c>
       <c r="E3" t="s" s="29">
         <v>6</v>
@@ -20905,21 +20900,21 @@
         <v>46</v>
       </c>
       <c r="H3" t="s" s="30">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="4" ht="14.7" customHeight="1">
       <c r="A4" t="s" s="19">
+        <v>200</v>
+      </c>
+      <c r="B4" t="s" s="27">
         <v>201</v>
       </c>
-      <c r="B4" t="s" s="27">
+      <c r="C4" t="s" s="27">
         <v>202</v>
       </c>
-      <c r="C4" t="s" s="27">
+      <c r="D4" t="s" s="27">
         <v>203</v>
-      </c>
-      <c r="D4" t="s" s="27">
-        <v>204</v>
       </c>
       <c r="E4" t="s" s="29">
         <v>6</v>
@@ -20931,7 +20926,7 @@
         <v>46</v>
       </c>
       <c r="H4" t="s" s="30">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="5" ht="13.65" customHeight="1">
@@ -30387,10 +30382,10 @@
   <sheetData>
     <row r="1" ht="13.2" customHeight="1">
       <c r="A1" t="s" s="32">
+        <v>204</v>
+      </c>
+      <c r="B1" t="s" s="32">
         <v>205</v>
-      </c>
-      <c r="B1" t="s" s="32">
-        <v>206</v>
       </c>
       <c r="C1" s="33"/>
       <c r="D1" s="33"/>
@@ -30398,7 +30393,7 @@
     </row>
     <row r="2" ht="13.2" customHeight="1">
       <c r="A2" t="s" s="34">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B2" t="s" s="35">
         <v>41</v>
@@ -30409,7 +30404,7 @@
     </row>
     <row r="3" ht="13" customHeight="1">
       <c r="A3" t="s" s="37">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B3" t="s" s="38">
         <v>49</v>
@@ -30420,7 +30415,7 @@
     </row>
     <row r="4" ht="13" customHeight="1">
       <c r="A4" t="s" s="37">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B4" t="s" s="38">
         <v>51</v>
@@ -30431,7 +30426,7 @@
     </row>
     <row r="5" ht="13" customHeight="1">
       <c r="A5" t="s" s="40">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B5" t="s" s="41">
         <v>53</v>
@@ -30442,10 +30437,10 @@
     </row>
     <row r="6" ht="13" customHeight="1">
       <c r="A6" t="s" s="37">
+        <v>163</v>
+      </c>
+      <c r="B6" t="s" s="40">
         <v>164</v>
-      </c>
-      <c r="B6" t="s" s="40">
-        <v>165</v>
       </c>
       <c r="C6" s="39"/>
       <c r="D6" s="39"/>
@@ -30453,7 +30448,7 @@
     </row>
     <row r="7" ht="13" customHeight="1">
       <c r="A7" t="s" s="37">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B7" t="s" s="38">
         <v>56</v>
@@ -30464,7 +30459,7 @@
     </row>
     <row r="8" ht="13" customHeight="1">
       <c r="A8" t="s" s="37">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B8" t="s" s="38">
         <v>60</v>
@@ -30475,7 +30470,7 @@
     </row>
     <row r="9" ht="13" customHeight="1">
       <c r="A9" t="s" s="37">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B9" t="s" s="38">
         <v>63</v>
@@ -30486,7 +30481,7 @@
     </row>
     <row r="10" ht="13" customHeight="1">
       <c r="A10" t="s" s="37">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B10" t="s" s="38">
         <v>65</v>
@@ -30497,7 +30492,7 @@
     </row>
     <row r="11" ht="13" customHeight="1">
       <c r="A11" t="s" s="37">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B11" t="s" s="38">
         <v>67</v>
@@ -30508,7 +30503,7 @@
     </row>
     <row r="12" ht="13" customHeight="1">
       <c r="A12" t="s" s="37">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B12" t="s" s="38">
         <v>70</v>
@@ -30519,7 +30514,7 @@
     </row>
     <row r="13" ht="13" customHeight="1">
       <c r="A13" t="s" s="37">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B13" t="s" s="38">
         <v>72</v>
@@ -30530,7 +30525,7 @@
     </row>
     <row r="14" ht="13" customHeight="1">
       <c r="A14" t="s" s="37">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B14" t="s" s="38">
         <v>74</v>
@@ -30541,7 +30536,7 @@
     </row>
     <row r="15" ht="13" customHeight="1">
       <c r="A15" t="s" s="37">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B15" t="s" s="38">
         <v>76</v>
@@ -30552,7 +30547,7 @@
     </row>
     <row r="16" ht="13" customHeight="1">
       <c r="A16" t="s" s="37">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B16" t="s" s="38">
         <v>80</v>
@@ -30563,7 +30558,7 @@
     </row>
     <row r="17" ht="13" customHeight="1">
       <c r="A17" t="s" s="37">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B17" t="s" s="38">
         <v>83</v>
@@ -30574,7 +30569,7 @@
     </row>
     <row r="18" ht="13" customHeight="1">
       <c r="A18" t="s" s="37">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B18" t="s" s="38">
         <v>85</v>
@@ -30585,7 +30580,7 @@
     </row>
     <row r="19" ht="13" customHeight="1">
       <c r="A19" t="s" s="37">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B19" t="s" s="38">
         <v>87</v>
@@ -30596,7 +30591,7 @@
     </row>
     <row r="20" ht="13" customHeight="1">
       <c r="A20" t="s" s="37">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B20" t="s" s="38">
         <v>89</v>
@@ -30607,10 +30602,10 @@
     </row>
     <row r="21" ht="13" customHeight="1">
       <c r="A21" t="s" s="37">
+        <v>156</v>
+      </c>
+      <c r="B21" t="s" s="38">
         <v>157</v>
-      </c>
-      <c r="B21" t="s" s="38">
-        <v>158</v>
       </c>
       <c r="C21" s="39"/>
       <c r="D21" s="39"/>
@@ -30618,7 +30613,7 @@
     </row>
     <row r="22" ht="13" customHeight="1">
       <c r="A22" t="s" s="37">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B22" t="s" s="38">
         <v>91</v>
@@ -30629,7 +30624,7 @@
     </row>
     <row r="23" ht="13" customHeight="1">
       <c r="A23" t="s" s="37">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B23" t="s" s="38">
         <v>94</v>
@@ -30640,7 +30635,7 @@
     </row>
     <row r="24" ht="13" customHeight="1">
       <c r="A24" t="s" s="37">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B24" t="s" s="38">
         <v>96</v>
@@ -30651,7 +30646,7 @@
     </row>
     <row r="25" ht="13" customHeight="1">
       <c r="A25" t="s" s="37">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B25" t="s" s="38">
         <v>98</v>
@@ -30662,7 +30657,7 @@
     </row>
     <row r="26" ht="13" customHeight="1">
       <c r="A26" t="s" s="37">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B26" t="s" s="38">
         <v>101</v>
@@ -30673,7 +30668,7 @@
     </row>
     <row r="27" ht="13" customHeight="1">
       <c r="A27" t="s" s="37">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B27" t="s" s="38">
         <v>103</v>
@@ -30684,10 +30679,10 @@
     </row>
     <row r="28" ht="13" customHeight="1">
       <c r="A28" t="s" s="37">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B28" t="s" s="38">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C28" s="39"/>
       <c r="D28" s="39"/>
@@ -30695,10 +30690,10 @@
     </row>
     <row r="29" ht="13" customHeight="1">
       <c r="A29" t="s" s="37">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B29" t="s" s="38">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C29" s="39"/>
       <c r="D29" s="39"/>
@@ -30706,10 +30701,10 @@
     </row>
     <row r="30" ht="13" customHeight="1">
       <c r="A30" t="s" s="37">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B30" t="s" s="38">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C30" s="39"/>
       <c r="D30" s="39"/>
@@ -30717,10 +30712,10 @@
     </row>
     <row r="31" ht="13" customHeight="1">
       <c r="A31" t="s" s="37">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B31" t="s" s="38">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C31" s="39"/>
       <c r="D31" s="39"/>
@@ -30728,10 +30723,10 @@
     </row>
     <row r="32" ht="13" customHeight="1">
       <c r="A32" t="s" s="37">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B32" t="s" s="38">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C32" s="39"/>
       <c r="D32" s="39"/>
@@ -30739,10 +30734,10 @@
     </row>
     <row r="33" ht="13" customHeight="1">
       <c r="A33" t="s" s="37">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B33" t="s" s="38">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C33" s="39"/>
       <c r="D33" s="39"/>
@@ -30750,10 +30745,10 @@
     </row>
     <row r="34" ht="13" customHeight="1">
       <c r="A34" t="s" s="37">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B34" t="s" s="38">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C34" s="39"/>
       <c r="D34" s="39"/>
@@ -30761,10 +30756,10 @@
     </row>
     <row r="35" ht="13" customHeight="1">
       <c r="A35" t="s" s="37">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B35" t="s" s="38">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C35" s="39"/>
       <c r="D35" s="39"/>
@@ -30772,10 +30767,10 @@
     </row>
     <row r="36" ht="13" customHeight="1">
       <c r="A36" t="s" s="37">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B36" t="s" s="38">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C36" s="39"/>
       <c r="D36" s="39"/>
@@ -30783,10 +30778,10 @@
     </row>
     <row r="37" ht="13" customHeight="1">
       <c r="A37" t="s" s="37">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B37" t="s" s="38">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C37" s="39"/>
       <c r="D37" s="39"/>
@@ -30794,10 +30789,10 @@
     </row>
     <row r="38" ht="13" customHeight="1">
       <c r="A38" t="s" s="37">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B38" t="s" s="38">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C38" s="39"/>
       <c r="D38" s="39"/>
@@ -30805,10 +30800,10 @@
     </row>
     <row r="39" ht="13" customHeight="1">
       <c r="A39" t="s" s="37">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B39" t="s" s="38">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C39" s="39"/>
       <c r="D39" s="39"/>
@@ -30816,10 +30811,10 @@
     </row>
     <row r="40" ht="13" customHeight="1">
       <c r="A40" t="s" s="37">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B40" t="s" s="38">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C40" s="39"/>
       <c r="D40" s="39"/>
@@ -30827,10 +30822,10 @@
     </row>
     <row r="41" ht="13" customHeight="1">
       <c r="A41" t="s" s="37">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B41" t="s" s="38">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C41" s="39"/>
       <c r="D41" s="39"/>
@@ -30838,10 +30833,10 @@
     </row>
     <row r="42" ht="13" customHeight="1">
       <c r="A42" t="s" s="37">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B42" t="s" s="38">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C42" s="39"/>
       <c r="D42" s="39"/>
@@ -30849,10 +30844,10 @@
     </row>
     <row r="43" ht="13" customHeight="1">
       <c r="A43" t="s" s="37">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B43" t="s" s="38">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C43" s="39"/>
       <c r="D43" s="39"/>
@@ -30860,10 +30855,10 @@
     </row>
     <row r="44" ht="13" customHeight="1">
       <c r="A44" t="s" s="37">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B44" t="s" s="38">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C44" s="39"/>
       <c r="D44" s="39"/>
@@ -30871,10 +30866,10 @@
     </row>
     <row r="45" ht="13" customHeight="1">
       <c r="A45" t="s" s="37">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B45" t="s" s="38">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C45" s="39"/>
       <c r="D45" s="39"/>
@@ -30882,10 +30877,10 @@
     </row>
     <row r="46" ht="13" customHeight="1">
       <c r="A46" t="s" s="37">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B46" t="s" s="38">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C46" s="39"/>
       <c r="D46" s="39"/>
@@ -30893,10 +30888,10 @@
     </row>
     <row r="47" ht="13" customHeight="1">
       <c r="A47" t="s" s="37">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B47" t="s" s="38">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C47" s="39"/>
       <c r="D47" s="39"/>
@@ -30904,10 +30899,10 @@
     </row>
     <row r="48" ht="13" customHeight="1">
       <c r="A48" t="s" s="42">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B48" t="s" s="38">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C48" s="39"/>
       <c r="D48" s="39"/>
@@ -30915,7 +30910,7 @@
     </row>
     <row r="49" ht="13" customHeight="1">
       <c r="A49" t="s" s="24">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B49" t="s" s="43">
         <v>49</v>
@@ -30926,7 +30921,7 @@
     </row>
     <row r="50" ht="13" customHeight="1">
       <c r="A50" t="s" s="2">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B50" t="s" s="43">
         <v>67</v>
@@ -30937,7 +30932,7 @@
     </row>
     <row r="51" ht="13" customHeight="1">
       <c r="A51" t="s" s="2">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B51" t="s" s="43">
         <v>83</v>
@@ -30948,7 +30943,7 @@
     </row>
     <row r="52" ht="13" customHeight="1">
       <c r="A52" t="s" s="2">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B52" t="s" s="43">
         <v>87</v>
@@ -30959,10 +30954,10 @@
     </row>
     <row r="53" ht="13" customHeight="1">
       <c r="A53" t="s" s="2">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B53" t="s" s="43">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C53" s="39"/>
       <c r="D53" s="39"/>
@@ -30970,7 +30965,7 @@
     </row>
     <row r="54" ht="13" customHeight="1">
       <c r="A54" t="s" s="2">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B54" t="s" s="43">
         <v>98</v>
@@ -30981,10 +30976,10 @@
     </row>
     <row r="55" ht="13" customHeight="1">
       <c r="A55" t="s" s="2">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B55" t="s" s="43">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C55" s="39"/>
       <c r="D55" s="39"/>
@@ -30992,10 +30987,10 @@
     </row>
     <row r="56" ht="13" customHeight="1">
       <c r="A56" t="s" s="2">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B56" t="s" s="43">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C56" s="39"/>
       <c r="D56" s="39"/>
@@ -31003,7 +30998,7 @@
     </row>
     <row r="57" ht="13" customHeight="1">
       <c r="A57" t="s" s="2">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B57" t="s" s="43">
         <v>101</v>
@@ -31014,10 +31009,10 @@
     </row>
     <row r="58" ht="13" customHeight="1">
       <c r="A58" t="s" s="2">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B58" t="s" s="43">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C58" s="39"/>
       <c r="D58" s="39"/>
@@ -31025,10 +31020,10 @@
     </row>
     <row r="59" ht="13" customHeight="1">
       <c r="A59" t="s" s="2">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B59" t="s" s="43">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C59" s="39"/>
       <c r="D59" s="39"/>
@@ -31036,10 +31031,10 @@
     </row>
     <row r="60" ht="13" customHeight="1">
       <c r="A60" t="s" s="2">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B60" t="s" s="43">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C60" s="39"/>
       <c r="D60" s="39"/>
@@ -31047,10 +31042,10 @@
     </row>
     <row r="61" ht="13" customHeight="1">
       <c r="A61" t="s" s="2">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B61" t="s" s="43">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C61" s="39"/>
       <c r="D61" s="39"/>
@@ -31058,10 +31053,10 @@
     </row>
     <row r="62" ht="13" customHeight="1">
       <c r="A62" t="s" s="2">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B62" t="s" s="43">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C62" s="39"/>
       <c r="D62" s="39"/>
@@ -31069,10 +31064,10 @@
     </row>
     <row r="63" ht="13" customHeight="1">
       <c r="A63" t="s" s="17">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B63" t="s" s="43">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C63" s="39"/>
       <c r="D63" s="39"/>
@@ -31080,10 +31075,10 @@
     </row>
     <row r="64" ht="13" customHeight="1">
       <c r="A64" t="s" s="24">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B64" t="s" s="44">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C64" s="39"/>
       <c r="D64" s="39"/>
@@ -31091,10 +31086,10 @@
     </row>
     <row r="65" ht="13" customHeight="1">
       <c r="A65" t="s" s="2">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B65" t="s" s="2">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C65" s="45"/>
       <c r="D65" s="39"/>
@@ -31102,10 +31097,10 @@
     </row>
     <row r="66" ht="13" customHeight="1">
       <c r="A66" t="s" s="2">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B66" t="s" s="2">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C66" s="45"/>
       <c r="D66" s="39"/>
@@ -31113,10 +31108,10 @@
     </row>
     <row r="67" ht="13" customHeight="1">
       <c r="A67" t="s" s="2">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B67" t="s" s="2">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C67" s="45"/>
       <c r="D67" s="39"/>
@@ -31124,10 +31119,10 @@
     </row>
     <row r="68" ht="13" customHeight="1">
       <c r="A68" t="s" s="2">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B68" t="s" s="2">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C68" s="45"/>
       <c r="D68" s="39"/>
@@ -31135,10 +31130,10 @@
     </row>
     <row r="69" ht="13" customHeight="1">
       <c r="A69" t="s" s="2">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B69" t="s" s="2">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C69" s="45"/>
       <c r="D69" s="39"/>
@@ -31146,10 +31141,10 @@
     </row>
     <row r="70" ht="13" customHeight="1">
       <c r="A70" t="s" s="2">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B70" t="s" s="2">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C70" s="45"/>
       <c r="D70" s="39"/>
@@ -31157,10 +31152,10 @@
     </row>
     <row r="71" ht="13" customHeight="1">
       <c r="A71" t="s" s="2">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B71" t="s" s="2">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="C71" s="45"/>
       <c r="D71" s="39"/>
@@ -31168,10 +31163,10 @@
     </row>
     <row r="72" ht="13" customHeight="1">
       <c r="A72" t="s" s="2">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B72" t="s" s="2">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C72" s="45"/>
       <c r="D72" s="39"/>
@@ -31211,22 +31206,22 @@
   <sheetData>
     <row r="1" ht="13.2" customHeight="1">
       <c r="A1" t="s" s="47">
+        <v>206</v>
+      </c>
+      <c r="B1" t="s" s="48">
         <v>207</v>
       </c>
-      <c r="B1" t="s" s="48">
+      <c r="C1" t="s" s="49">
         <v>208</v>
       </c>
-      <c r="C1" t="s" s="49">
+      <c r="D1" t="s" s="32">
         <v>209</v>
       </c>
-      <c r="D1" t="s" s="32">
+      <c r="E1" t="s" s="32">
         <v>210</v>
       </c>
-      <c r="E1" t="s" s="32">
+      <c r="F1" t="s" s="32">
         <v>211</v>
-      </c>
-      <c r="F1" t="s" s="32">
-        <v>212</v>
       </c>
     </row>
     <row r="2" ht="13.2" customHeight="1">
@@ -31234,19 +31229,19 @@
         <v>41</v>
       </c>
       <c r="B2" t="s" s="51">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C2" t="s" s="51">
         <v>49</v>
       </c>
       <c r="D2" t="s" s="52">
+        <v>213</v>
+      </c>
+      <c r="E2" t="s" s="52">
         <v>214</v>
       </c>
-      <c r="E2" t="s" s="52">
-        <v>215</v>
-      </c>
       <c r="F2" t="s" s="53">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="3" ht="13" customHeight="1">
@@ -31254,19 +31249,19 @@
         <v>41</v>
       </c>
       <c r="B3" t="s" s="51">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C3" t="s" s="51">
         <v>51</v>
       </c>
       <c r="D3" t="s" s="54">
+        <v>213</v>
+      </c>
+      <c r="E3" t="s" s="54">
         <v>214</v>
       </c>
-      <c r="E3" t="s" s="54">
-        <v>215</v>
-      </c>
       <c r="F3" t="s" s="55">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="4" ht="13" customHeight="1">
@@ -31274,19 +31269,19 @@
         <v>41</v>
       </c>
       <c r="B4" t="s" s="51">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C4" t="s" s="51">
         <v>53</v>
       </c>
       <c r="D4" t="s" s="54">
+        <v>213</v>
+      </c>
+      <c r="E4" t="s" s="54">
         <v>214</v>
       </c>
-      <c r="E4" t="s" s="54">
-        <v>215</v>
-      </c>
       <c r="F4" t="s" s="55">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="5" ht="13" customHeight="1">
@@ -31294,19 +31289,19 @@
         <v>41</v>
       </c>
       <c r="B5" t="s" s="51">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C5" t="s" s="51">
         <v>85</v>
       </c>
       <c r="D5" t="s" s="54">
+        <v>213</v>
+      </c>
+      <c r="E5" t="s" s="54">
         <v>214</v>
       </c>
-      <c r="E5" t="s" s="54">
-        <v>215</v>
-      </c>
       <c r="F5" t="s" s="55">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="6" ht="13" customHeight="1">
@@ -31314,19 +31309,19 @@
         <v>41</v>
       </c>
       <c r="B6" t="s" s="51">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C6" t="s" s="51">
         <v>94</v>
       </c>
       <c r="D6" t="s" s="54">
+        <v>213</v>
+      </c>
+      <c r="E6" t="s" s="54">
         <v>214</v>
       </c>
-      <c r="E6" t="s" s="54">
-        <v>215</v>
-      </c>
       <c r="F6" t="s" s="55">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="7" ht="13" customHeight="1">
@@ -31334,19 +31329,19 @@
         <v>41</v>
       </c>
       <c r="B7" t="s" s="51">
+        <v>212</v>
+      </c>
+      <c r="C7" t="s" s="51">
+        <v>150</v>
+      </c>
+      <c r="D7" t="s" s="54">
         <v>213</v>
       </c>
-      <c r="C7" t="s" s="51">
-        <v>151</v>
-      </c>
-      <c r="D7" t="s" s="54">
+      <c r="E7" t="s" s="54">
         <v>214</v>
       </c>
-      <c r="E7" t="s" s="54">
-        <v>215</v>
-      </c>
       <c r="F7" t="s" s="55">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="8" ht="13" customHeight="1">
@@ -31354,19 +31349,19 @@
         <v>41</v>
       </c>
       <c r="B8" t="s" s="51">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C8" t="s" s="51">
         <v>87</v>
       </c>
       <c r="D8" t="s" s="54">
+        <v>213</v>
+      </c>
+      <c r="E8" t="s" s="54">
         <v>214</v>
       </c>
-      <c r="E8" t="s" s="54">
-        <v>215</v>
-      </c>
       <c r="F8" t="s" s="55">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="9" ht="13" customHeight="1">
@@ -31374,19 +31369,19 @@
         <v>41</v>
       </c>
       <c r="B9" t="s" s="51">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C9" t="s" s="51">
         <v>101</v>
       </c>
       <c r="D9" t="s" s="54">
+        <v>213</v>
+      </c>
+      <c r="E9" t="s" s="54">
         <v>214</v>
       </c>
-      <c r="E9" t="s" s="54">
-        <v>215</v>
-      </c>
       <c r="F9" t="s" s="55">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="10" ht="13" customHeight="1">
@@ -31394,39 +31389,39 @@
         <v>41</v>
       </c>
       <c r="B10" t="s" s="51">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C10" t="s" s="51">
         <v>103</v>
       </c>
       <c r="D10" t="s" s="54">
+        <v>213</v>
+      </c>
+      <c r="E10" t="s" s="54">
         <v>214</v>
       </c>
-      <c r="E10" t="s" s="54">
-        <v>215</v>
-      </c>
       <c r="F10" t="s" s="55">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="11" ht="13" customHeight="1">
       <c r="A11" t="s" s="50">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B11" t="s" s="51">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C11" t="s" s="51">
         <v>41</v>
       </c>
       <c r="D11" t="s" s="54">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="E11" t="s" s="54">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="F11" t="s" s="55">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="12" ht="13" customHeight="1">
@@ -31434,19 +31429,19 @@
         <v>41</v>
       </c>
       <c r="B12" t="s" s="51">
+        <v>212</v>
+      </c>
+      <c r="C12" t="s" s="51">
+        <v>113</v>
+      </c>
+      <c r="D12" t="s" s="54">
         <v>213</v>
       </c>
-      <c r="C12" t="s" s="51">
-        <v>114</v>
-      </c>
-      <c r="D12" t="s" s="54">
+      <c r="E12" t="s" s="54">
         <v>214</v>
       </c>
-      <c r="E12" t="s" s="54">
-        <v>215</v>
-      </c>
       <c r="F12" t="s" s="55">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="13" ht="13" customHeight="1">
@@ -31454,19 +31449,19 @@
         <v>41</v>
       </c>
       <c r="B13" t="s" s="51">
+        <v>212</v>
+      </c>
+      <c r="C13" t="s" s="51">
+        <v>130</v>
+      </c>
+      <c r="D13" t="s" s="54">
         <v>213</v>
       </c>
-      <c r="C13" t="s" s="51">
-        <v>131</v>
-      </c>
-      <c r="D13" t="s" s="54">
+      <c r="E13" t="s" s="54">
         <v>214</v>
       </c>
-      <c r="E13" t="s" s="54">
-        <v>215</v>
-      </c>
       <c r="F13" t="s" s="55">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="14" ht="13" customHeight="1">
@@ -31474,19 +31469,19 @@
         <v>74</v>
       </c>
       <c r="B14" t="s" s="51">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C14" t="s" s="51">
         <v>49</v>
       </c>
       <c r="D14" t="s" s="54">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="E14" t="s" s="54">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="F14" t="s" s="55">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="15" ht="13" customHeight="1">
@@ -31494,19 +31489,19 @@
         <v>41</v>
       </c>
       <c r="B15" t="s" s="51">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C15" t="s" s="51">
         <v>49</v>
       </c>
       <c r="D15" t="s" s="54">
+        <v>213</v>
+      </c>
+      <c r="E15" t="s" s="54">
         <v>214</v>
       </c>
-      <c r="E15" t="s" s="54">
-        <v>215</v>
-      </c>
       <c r="F15" t="s" s="55">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="16" ht="13" customHeight="1">
@@ -31514,19 +31509,19 @@
         <v>51</v>
       </c>
       <c r="B16" t="s" s="51">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C16" t="s" s="51">
         <v>49</v>
       </c>
       <c r="D16" t="s" s="54">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="E16" t="s" s="54">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="F16" t="s" s="55">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="17" ht="13" customHeight="1">
@@ -31534,19 +31529,19 @@
         <v>53</v>
       </c>
       <c r="B17" t="s" s="51">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C17" t="s" s="51">
         <v>49</v>
       </c>
       <c r="D17" t="s" s="54">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="E17" t="s" s="54">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="F17" t="s" s="55">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="18" ht="13" customHeight="1">
@@ -31554,19 +31549,19 @@
         <v>76</v>
       </c>
       <c r="B18" t="s" s="51">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C18" t="s" s="51">
         <v>49</v>
       </c>
       <c r="D18" t="s" s="54">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="E18" t="s" s="54">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="F18" t="s" s="55">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="19" ht="13" customHeight="1">
@@ -31574,19 +31569,19 @@
         <v>85</v>
       </c>
       <c r="B19" t="s" s="51">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C19" t="s" s="51">
         <v>49</v>
       </c>
       <c r="D19" t="s" s="54">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="E19" t="s" s="54">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="F19" t="s" s="55">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="20" ht="13" customHeight="1">
@@ -31594,19 +31589,19 @@
         <v>89</v>
       </c>
       <c r="B20" t="s" s="51">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C20" t="s" s="51">
         <v>49</v>
       </c>
       <c r="D20" t="s" s="54">
+        <v>213</v>
+      </c>
+      <c r="E20" t="s" s="54">
         <v>214</v>
       </c>
-      <c r="E20" t="s" s="54">
-        <v>215</v>
-      </c>
       <c r="F20" t="s" s="55">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="21" ht="13" customHeight="1">
@@ -31614,19 +31609,19 @@
         <v>49</v>
       </c>
       <c r="B21" t="s" s="57">
+        <v>212</v>
+      </c>
+      <c r="C21" t="s" s="57">
+        <v>142</v>
+      </c>
+      <c r="D21" t="s" s="58">
         <v>213</v>
       </c>
-      <c r="C21" t="s" s="57">
-        <v>143</v>
-      </c>
-      <c r="D21" t="s" s="58">
+      <c r="E21" t="s" s="58">
         <v>214</v>
       </c>
-      <c r="E21" t="s" s="58">
-        <v>215</v>
-      </c>
       <c r="F21" t="s" s="59">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
   </sheetData>
@@ -31654,31 +31649,31 @@
   <sheetData>
     <row r="1" ht="13.45" customHeight="1">
       <c r="A1" t="s" s="61">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B1" t="s" s="62">
         <v>27</v>
       </c>
       <c r="C1" t="s" s="62">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="D1" t="s" s="62">
         <v>29</v>
       </c>
       <c r="E1" t="s" s="62">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="F1" t="s" s="62">
         <v>28</v>
       </c>
       <c r="G1" t="s" s="62">
+        <v>219</v>
+      </c>
+      <c r="H1" t="s" s="62">
         <v>220</v>
       </c>
-      <c r="H1" t="s" s="62">
+      <c r="I1" t="s" s="62">
         <v>221</v>
-      </c>
-      <c r="I1" t="s" s="62">
-        <v>222</v>
       </c>
     </row>
     <row r="2" ht="13.65" customHeight="1">
@@ -31686,19 +31681,19 @@
         <v>48</v>
       </c>
       <c r="B2" t="s" s="63">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="C2" s="64">
         <v>1</v>
       </c>
       <c r="D2" t="s" s="65">
+        <v>223</v>
+      </c>
+      <c r="E2" t="s" s="65">
         <v>224</v>
       </c>
-      <c r="E2" t="s" s="65">
+      <c r="F2" t="s" s="65">
         <v>225</v>
-      </c>
-      <c r="F2" t="s" s="65">
-        <v>226</v>
       </c>
       <c r="G2" s="64">
         <v>-150</v>
@@ -31715,19 +31710,19 @@
         <v>48</v>
       </c>
       <c r="B3" t="s" s="66">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="C3" s="67">
         <v>2</v>
       </c>
       <c r="D3" t="s" s="68">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="E3" t="s" s="68">
+        <v>227</v>
+      </c>
+      <c r="F3" t="s" s="68">
         <v>228</v>
-      </c>
-      <c r="F3" t="s" s="68">
-        <v>229</v>
       </c>
       <c r="G3" s="67">
         <v>-10</v>
@@ -31744,19 +31739,19 @@
         <v>48</v>
       </c>
       <c r="B4" t="s" s="66">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="C4" s="67">
         <v>3</v>
       </c>
       <c r="D4" t="s" s="68">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="E4" t="s" s="68">
+        <v>230</v>
+      </c>
+      <c r="F4" t="s" s="68">
         <v>231</v>
-      </c>
-      <c r="F4" t="s" s="68">
-        <v>232</v>
       </c>
       <c r="G4" s="67">
         <v>15</v>
@@ -31773,19 +31768,19 @@
         <v>48</v>
       </c>
       <c r="B5" t="s" s="66">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="C5" s="67">
         <v>4</v>
       </c>
       <c r="D5" t="s" s="68">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="E5" t="s" s="68">
+        <v>233</v>
+      </c>
+      <c r="F5" t="s" s="68">
         <v>234</v>
-      </c>
-      <c r="F5" t="s" s="68">
-        <v>235</v>
       </c>
       <c r="G5" s="67">
         <v>50</v>
@@ -31802,19 +31797,19 @@
         <v>48</v>
       </c>
       <c r="B6" t="s" s="66">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="C6" s="67">
         <v>5</v>
       </c>
       <c r="D6" t="s" s="68">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="E6" t="s" s="68">
+        <v>236</v>
+      </c>
+      <c r="F6" t="s" s="68">
         <v>237</v>
-      </c>
-      <c r="F6" t="s" s="68">
-        <v>238</v>
       </c>
       <c r="G6" s="67">
         <v>90</v>
@@ -31823,7 +31818,7 @@
         <v>150</v>
       </c>
       <c r="I6" t="s" s="68">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="7" ht="13.65" customHeight="1">
@@ -31831,19 +31826,19 @@
         <v>48</v>
       </c>
       <c r="B7" t="s" s="66">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="C7" s="67">
         <v>6</v>
       </c>
       <c r="D7" t="s" s="68">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="E7" t="s" s="68">
+        <v>240</v>
+      </c>
+      <c r="F7" t="s" s="68">
         <v>241</v>
-      </c>
-      <c r="F7" t="s" s="68">
-        <v>242</v>
       </c>
       <c r="G7" s="67">
         <v>140</v>
@@ -31860,19 +31855,19 @@
         <v>48</v>
       </c>
       <c r="B8" t="s" s="66">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C8" s="67">
         <v>7</v>
       </c>
       <c r="D8" t="s" s="68">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="E8" t="s" s="68">
+        <v>243</v>
+      </c>
+      <c r="F8" t="s" s="68">
         <v>244</v>
-      </c>
-      <c r="F8" t="s" s="68">
-        <v>245</v>
       </c>
       <c r="G8" s="67">
         <v>501</v>
@@ -31889,19 +31884,19 @@
         <v>48</v>
       </c>
       <c r="B9" t="s" s="66">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="C9" s="67">
         <v>8</v>
       </c>
       <c r="D9" t="s" s="68">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="E9" t="s" s="68">
+        <v>246</v>
+      </c>
+      <c r="F9" t="s" s="68">
         <v>247</v>
-      </c>
-      <c r="F9" t="s" s="68">
-        <v>248</v>
       </c>
       <c r="G9" s="67">
         <v>1500</v>
@@ -31918,19 +31913,19 @@
         <v>48</v>
       </c>
       <c r="B10" t="s" s="66">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C10" s="67">
         <v>9</v>
       </c>
       <c r="D10" t="s" s="68">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="E10" t="s" s="68">
+        <v>249</v>
+      </c>
+      <c r="F10" t="s" s="68">
         <v>250</v>
-      </c>
-      <c r="F10" t="s" s="68">
-        <v>251</v>
       </c>
       <c r="G10" s="67">
         <v>1828</v>

</xml_diff>

<commit_message>
feat - import sans uri
</commit_message>
<xml_diff>
--- a/src/main/resources/datasets/Import_Chartres_Projet.xlsx
+++ b/src/main/resources/datasets/Import_Chartres_Projet.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="259">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="285" count="220">
   <si>
     <t>Nom</t>
   </si>
@@ -1002,6 +1002,84 @@
   </si>
   <si>
     <t>retour progressif du bâti après une longue phase de culture de la vigne du coteau. Transformation du coteau dès 1840 dans le cadre des travaux ferroviaires de Chartres. Châteaux d’eau successifs et trois maisons d’habitation sont construits sur ces terrains propriétés de RFF jusqu’en 2013. terrains libérés de toute construction en 2013 et diagnostiqués. Terrains fouillés en 2015.</t>
+  </si>
+  <si>
+    <t>UE</t>
+  </si>
+  <si>
+    <t>Type Label</t>
+  </si>
+  <si>
+    <t>Unité élémentaire</t>
+  </si>
+  <si>
+    <t>Subdivision</t>
+  </si>
+  <si>
+    <t>EA</t>
+  </si>
+  <si>
+    <t>EAS</t>
+  </si>
+  <si>
+    <t>Cycle Label</t>
+  </si>
+  <si>
+    <t>Dépôt</t>
+  </si>
+  <si>
+    <t>Erosion</t>
+  </si>
+  <si>
+    <t>Agent Label</t>
+  </si>
+  <si>
+    <t>Interpretation Label</t>
+  </si>
+  <si>
+    <t>Terre végétale</t>
+  </si>
+  <si>
+    <t>Autre dépôt</t>
+  </si>
+  <si>
+    <t>Remblai</t>
+  </si>
+  <si>
+    <t>Comblement</t>
+  </si>
+  <si>
+    <t>Mur</t>
+  </si>
+  <si>
+    <t>Interprétation normalisée</t>
+  </si>
+  <si>
+    <t>Couche d'occupation</t>
+  </si>
+  <si>
+    <t>Couche de démolition</t>
+  </si>
+  <si>
+    <t>Canalisation</t>
+  </si>
+  <si>
+    <t>Filin</t>
+  </si>
+  <si>
+    <t>Parcelle</t>
+  </si>
+  <si>
+    <t>Commune</t>
+  </si>
+  <si>
+    <t>Relation Label</t>
+  </si>
+  <si>
+    <t>postérieur à</t>
+  </si>
+  <si>
+    <t>antérieur à</t>
   </si>
 </sst>
 </file>
@@ -3155,15 +3233,15 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr defaultColWidth="12.6667" defaultRowHeight="15.75" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="18" style="1" customWidth="1"/>
-    <col min="2" max="2" width="37.8516" style="1" customWidth="1"/>
-    <col min="3" max="3" width="12.6719" style="1" customWidth="1"/>
-    <col min="4" max="4" width="115.352" style="1" customWidth="1"/>
-    <col min="5" max="5" width="12.6719" style="1" customWidth="1"/>
-    <col min="6" max="16384" width="12.6719" style="1" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" style="1" width="18.0"/>
+    <col min="2" max="2" customWidth="true" style="1" width="37.8516"/>
+    <col min="3" max="3" customWidth="true" style="1" width="12.6719"/>
+    <col min="4" max="4" customWidth="true" style="1" width="115.352"/>
+    <col min="5" max="5" customWidth="true" style="1" width="12.6719"/>
+    <col min="6" max="16384" customWidth="true" style="1" width="12.6719"/>
   </cols>
   <sheetData>
     <row r="1" ht="13.65" customHeight="1">
@@ -3180,248 +3258,267 @@
         <v>3</v>
       </c>
       <c r="E1" s="3"/>
+      <c r="F1" t="s" s="1">
+        <v>260</v>
+      </c>
     </row>
     <row r="2" ht="15.35" customHeight="1">
       <c r="A2" t="s" s="2">
         <v>4</v>
       </c>
-      <c r="B2" t="s" s="4">
-        <v>5</v>
-      </c>
+      <c r="B2" s="4"/>
       <c r="C2" t="s" s="5">
         <v>6</v>
       </c>
       <c r="D2" s="6"/>
       <c r="E2" s="7"/>
+      <c r="F2" t="s" s="1">
+        <v>280</v>
+      </c>
     </row>
     <row r="3" ht="15.35" customHeight="1">
       <c r="A3" t="s" s="2">
         <v>7</v>
       </c>
-      <c r="B3" t="s" s="4">
-        <v>5</v>
-      </c>
+      <c r="B3" s="4"/>
       <c r="C3" t="s" s="5">
         <v>6</v>
       </c>
       <c r="D3" s="6"/>
       <c r="E3" s="7"/>
+      <c r="F3" t="s" s="1">
+        <v>280</v>
+      </c>
     </row>
     <row r="4" ht="15.35" customHeight="1">
       <c r="A4" t="s" s="2">
         <v>8</v>
       </c>
-      <c r="B4" t="s" s="4">
-        <v>5</v>
-      </c>
+      <c r="B4" s="4"/>
       <c r="C4" t="s" s="5">
         <v>6</v>
       </c>
       <c r="D4" s="6"/>
       <c r="E4" s="7"/>
+      <c r="F4" t="s" s="1">
+        <v>280</v>
+      </c>
     </row>
     <row r="5" ht="15.35" customHeight="1">
       <c r="A5" t="s" s="2">
         <v>9</v>
       </c>
-      <c r="B5" t="s" s="4">
-        <v>5</v>
-      </c>
+      <c r="B5" s="4"/>
       <c r="C5" t="s" s="5">
         <v>6</v>
       </c>
       <c r="D5" s="6"/>
       <c r="E5" s="7"/>
+      <c r="F5" t="s" s="1">
+        <v>280</v>
+      </c>
     </row>
     <row r="6" ht="15.35" customHeight="1">
       <c r="A6" t="s" s="2">
         <v>10</v>
       </c>
-      <c r="B6" t="s" s="4">
-        <v>5</v>
-      </c>
+      <c r="B6" s="4"/>
       <c r="C6" t="s" s="5">
         <v>6</v>
       </c>
       <c r="D6" s="6"/>
       <c r="E6" s="7"/>
+      <c r="F6" t="s" s="1">
+        <v>280</v>
+      </c>
     </row>
     <row r="7" ht="15.35" customHeight="1">
       <c r="A7" t="s" s="2">
         <v>11</v>
       </c>
-      <c r="B7" t="s" s="4">
-        <v>5</v>
-      </c>
+      <c r="B7" s="4"/>
       <c r="C7" t="s" s="5">
         <v>6</v>
       </c>
       <c r="D7" s="6"/>
       <c r="E7" s="7"/>
+      <c r="F7" t="s" s="1">
+        <v>280</v>
+      </c>
     </row>
     <row r="8" ht="15.35" customHeight="1">
       <c r="A8" t="s" s="2">
         <v>12</v>
       </c>
-      <c r="B8" t="s" s="4">
-        <v>5</v>
-      </c>
+      <c r="B8" s="4"/>
       <c r="C8" t="s" s="5">
         <v>6</v>
       </c>
       <c r="D8" s="6"/>
       <c r="E8" s="7"/>
+      <c r="F8" t="s" s="1">
+        <v>280</v>
+      </c>
     </row>
     <row r="9" ht="15.35" customHeight="1">
       <c r="A9" t="s" s="2">
         <v>13</v>
       </c>
-      <c r="B9" t="s" s="4">
-        <v>5</v>
-      </c>
+      <c r="B9" s="4"/>
       <c r="C9" t="s" s="5">
         <v>6</v>
       </c>
       <c r="D9" s="6"/>
       <c r="E9" s="7"/>
+      <c r="F9" t="s" s="1">
+        <v>280</v>
+      </c>
     </row>
     <row r="10" ht="15.35" customHeight="1">
       <c r="A10" t="s" s="2">
         <v>14</v>
       </c>
-      <c r="B10" t="s" s="4">
-        <v>5</v>
-      </c>
+      <c r="B10" s="4"/>
       <c r="C10" t="s" s="5">
         <v>6</v>
       </c>
       <c r="D10" s="6"/>
       <c r="E10" s="7"/>
+      <c r="F10" t="s" s="1">
+        <v>280</v>
+      </c>
     </row>
     <row r="11" ht="15.35" customHeight="1">
       <c r="A11" t="s" s="2">
         <v>15</v>
       </c>
-      <c r="B11" t="s" s="4">
-        <v>5</v>
-      </c>
+      <c r="B11" s="4"/>
       <c r="C11" t="s" s="5">
         <v>6</v>
       </c>
       <c r="D11" s="6"/>
       <c r="E11" s="7"/>
+      <c r="F11" t="s" s="1">
+        <v>280</v>
+      </c>
     </row>
     <row r="12" ht="15.35" customHeight="1">
       <c r="A12" t="s" s="2">
         <v>16</v>
       </c>
-      <c r="B12" t="s" s="4">
-        <v>5</v>
-      </c>
+      <c r="B12" s="4"/>
       <c r="C12" t="s" s="5">
         <v>6</v>
       </c>
       <c r="D12" s="6"/>
       <c r="E12" s="7"/>
+      <c r="F12" t="s" s="1">
+        <v>280</v>
+      </c>
     </row>
     <row r="13" ht="15.35" customHeight="1">
       <c r="A13" t="s" s="2">
         <v>17</v>
       </c>
-      <c r="B13" t="s" s="4">
-        <v>5</v>
-      </c>
+      <c r="B13" s="4"/>
       <c r="C13" t="s" s="5">
         <v>6</v>
       </c>
       <c r="D13" s="6"/>
       <c r="E13" s="7"/>
+      <c r="F13" t="s" s="1">
+        <v>280</v>
+      </c>
     </row>
     <row r="14" ht="15.35" customHeight="1">
       <c r="A14" t="s" s="2">
         <v>18</v>
       </c>
-      <c r="B14" t="s" s="4">
-        <v>5</v>
-      </c>
+      <c r="B14" s="4"/>
       <c r="C14" t="s" s="5">
         <v>6</v>
       </c>
       <c r="D14" s="6"/>
       <c r="E14" s="7"/>
+      <c r="F14" t="s" s="1">
+        <v>280</v>
+      </c>
     </row>
     <row r="15" ht="15.35" customHeight="1">
       <c r="A15" t="s" s="2">
         <v>19</v>
       </c>
-      <c r="B15" t="s" s="4">
-        <v>5</v>
-      </c>
+      <c r="B15" s="4"/>
       <c r="C15" t="s" s="5">
         <v>6</v>
       </c>
       <c r="D15" s="6"/>
       <c r="E15" s="7"/>
+      <c r="F15" t="s" s="1">
+        <v>280</v>
+      </c>
     </row>
     <row r="16" ht="15.35" customHeight="1">
       <c r="A16" t="s" s="2">
         <v>20</v>
       </c>
-      <c r="B16" t="s" s="4">
-        <v>5</v>
-      </c>
+      <c r="B16" s="4"/>
       <c r="C16" t="s" s="5">
         <v>6</v>
       </c>
       <c r="D16" s="6"/>
       <c r="E16" s="7"/>
+      <c r="F16" t="s" s="1">
+        <v>280</v>
+      </c>
     </row>
     <row r="17" ht="15.35" customHeight="1">
       <c r="A17" t="s" s="2">
         <v>21</v>
       </c>
-      <c r="B17" t="s" s="4">
-        <v>5</v>
-      </c>
+      <c r="B17" s="4"/>
       <c r="C17" t="s" s="5">
         <v>6</v>
       </c>
       <c r="D17" s="6"/>
       <c r="E17" s="7"/>
+      <c r="F17" t="s" s="1">
+        <v>280</v>
+      </c>
     </row>
     <row r="18" ht="15.35" customHeight="1">
       <c r="A18" t="s" s="2">
         <v>22</v>
       </c>
-      <c r="B18" t="s" s="4">
-        <v>5</v>
-      </c>
+      <c r="B18" s="4"/>
       <c r="C18" t="s" s="5">
         <v>6</v>
       </c>
       <c r="D18" s="6"/>
       <c r="E18" s="7"/>
+      <c r="F18" t="s" s="1">
+        <v>280</v>
+      </c>
     </row>
     <row r="19" ht="15.35" customHeight="1">
       <c r="A19" t="s" s="2">
         <v>23</v>
       </c>
-      <c r="B19" t="s" s="4">
-        <v>5</v>
-      </c>
+      <c r="B19" s="4"/>
       <c r="C19" t="s" s="5">
         <v>6</v>
       </c>
       <c r="D19" s="6"/>
       <c r="E19" s="7"/>
+      <c r="F19" t="s" s="1">
+        <v>280</v>
+      </c>
     </row>
     <row r="20" ht="15.35" customHeight="1">
       <c r="A20" t="s" s="2">
         <v>24</v>
       </c>
-      <c r="B20" t="s" s="4">
-        <v>25</v>
-      </c>
+      <c r="B20" s="4"/>
       <c r="C20" t="s" s="5">
         <v>6</v>
       </c>
@@ -3429,6 +3526,9 @@
         <v>26</v>
       </c>
       <c r="E20" s="8"/>
+      <c r="F20" t="s" s="1">
+        <v>281</v>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>
@@ -3465,11 +3565,11 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:E11"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr defaultColWidth="16.3333" defaultRowHeight="13.45" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="5" width="16.3516" style="9" customWidth="1"/>
-    <col min="6" max="16384" width="16.3516" style="9" customWidth="1"/>
+    <col min="1" max="5" customWidth="true" style="9" width="16.3516"/>
+    <col min="6" max="16384" customWidth="true" style="9" width="16.3516"/>
   </cols>
   <sheetData>
     <row r="1" ht="15.55" customHeight="1">
@@ -3501,7 +3601,7 @@
         <v>32</v>
       </c>
       <c r="B3" t="s" s="14">
-        <v>33</v>
+        <v>259</v>
       </c>
       <c r="C3" s="15"/>
       <c r="D3" s="16"/>
@@ -3512,7 +3612,7 @@
         <v>32</v>
       </c>
       <c r="B4" t="s" s="19">
-        <v>33</v>
+        <v>259</v>
       </c>
       <c r="C4" t="s" s="20">
         <v>34</v>
@@ -3588,22 +3688,22 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N998"/>
+  <dimension ref="A1:R998"/>
   <sheetFormatPr defaultColWidth="12.6667" defaultRowHeight="15.75" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="12.6719" style="30" customWidth="1"/>
-    <col min="2" max="2" width="35.3516" style="30" customWidth="1"/>
-    <col min="3" max="3" width="53.1719" style="30" customWidth="1"/>
-    <col min="4" max="4" width="44.8516" style="30" customWidth="1"/>
-    <col min="5" max="5" width="12.6719" style="30" customWidth="1"/>
-    <col min="6" max="6" width="40.3516" style="30" customWidth="1"/>
-    <col min="7" max="7" width="23.5" style="30" customWidth="1"/>
-    <col min="8" max="8" width="12.6719" style="30" customWidth="1"/>
-    <col min="9" max="9" width="45.6719" style="30" customWidth="1"/>
-    <col min="10" max="10" width="14.8516" style="30" customWidth="1"/>
-    <col min="11" max="11" width="15.5" style="30" customWidth="1"/>
-    <col min="12" max="14" width="12.6719" style="30" customWidth="1"/>
-    <col min="15" max="16384" width="12.6719" style="30" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" style="30" width="12.6719"/>
+    <col min="2" max="2" customWidth="true" style="30" width="35.3516"/>
+    <col min="3" max="3" customWidth="true" style="30" width="53.1719"/>
+    <col min="4" max="4" customWidth="true" style="30" width="44.8516"/>
+    <col min="5" max="5" customWidth="true" style="30" width="12.6719"/>
+    <col min="6" max="6" customWidth="true" style="30" width="40.3516"/>
+    <col min="7" max="7" customWidth="true" style="30" width="23.5"/>
+    <col min="8" max="8" customWidth="true" style="30" width="12.6719"/>
+    <col min="9" max="9" customWidth="true" style="30" width="45.6719"/>
+    <col min="10" max="10" customWidth="true" style="30" width="14.8516"/>
+    <col min="11" max="11" customWidth="true" style="30" width="15.5"/>
+    <col min="12" max="14" customWidth="true" style="30" width="12.6719"/>
+    <col min="15" max="16384" customWidth="true" style="30" width="12.6719"/>
   </cols>
   <sheetData>
     <row r="1" ht="13.65" customHeight="1">
@@ -3649,6 +3749,18 @@
       <c r="N1" t="s" s="32">
         <v>48</v>
       </c>
+      <c r="O1" t="s" s="30">
+        <v>260</v>
+      </c>
+      <c r="P1" t="s" s="30">
+        <v>265</v>
+      </c>
+      <c r="Q1" t="s" s="30">
+        <v>268</v>
+      </c>
+      <c r="R1" t="s" s="30">
+        <v>269</v>
+      </c>
     </row>
     <row r="2" ht="13.75" customHeight="1">
       <c r="A2" t="s" s="2">
@@ -3657,16 +3769,10 @@
       <c r="B2" t="s" s="2">
         <v>50</v>
       </c>
-      <c r="C2" t="s" s="33">
-        <v>51</v>
-      </c>
-      <c r="D2" t="s" s="33">
-        <v>52</v>
-      </c>
+      <c r="C2" s="33"/>
+      <c r="D2" s="33"/>
       <c r="E2" s="34"/>
-      <c r="F2" t="s" s="35">
-        <v>53</v>
-      </c>
+      <c r="F2" s="35"/>
       <c r="G2" t="s" s="5">
         <v>54</v>
       </c>
@@ -3687,6 +3793,15 @@
       <c r="N2" s="37">
         <v>9</v>
       </c>
+      <c r="O2" t="s" s="30">
+        <v>261</v>
+      </c>
+      <c r="P2" t="s" s="30">
+        <v>266</v>
+      </c>
+      <c r="R2" t="s" s="30">
+        <v>270</v>
+      </c>
     </row>
     <row r="3" ht="13.75" customHeight="1">
       <c r="A3" t="s" s="2">
@@ -3695,16 +3810,10 @@
       <c r="B3" t="s" s="2">
         <v>58</v>
       </c>
-      <c r="C3" t="s" s="33">
-        <v>51</v>
-      </c>
-      <c r="D3" t="s" s="33">
-        <v>52</v>
-      </c>
+      <c r="C3" s="33"/>
+      <c r="D3" s="33"/>
       <c r="E3" s="34"/>
-      <c r="F3" t="s" s="35">
-        <v>53</v>
-      </c>
+      <c r="F3" s="35"/>
       <c r="G3" t="s" s="5">
         <v>54</v>
       </c>
@@ -3725,6 +3834,15 @@
       <c r="N3" s="37">
         <v>8</v>
       </c>
+      <c r="O3" t="s" s="30">
+        <v>261</v>
+      </c>
+      <c r="P3" t="s" s="30">
+        <v>266</v>
+      </c>
+      <c r="R3" t="s" s="30">
+        <v>270</v>
+      </c>
     </row>
     <row r="4" ht="13.75" customHeight="1">
       <c r="A4" t="s" s="2">
@@ -3733,16 +3851,10 @@
       <c r="B4" t="s" s="2">
         <v>60</v>
       </c>
-      <c r="C4" t="s" s="33">
-        <v>51</v>
-      </c>
-      <c r="D4" t="s" s="33">
-        <v>52</v>
-      </c>
+      <c r="C4" s="33"/>
+      <c r="D4" s="33"/>
       <c r="E4" s="34"/>
-      <c r="F4" t="s" s="35">
-        <v>53</v>
-      </c>
+      <c r="F4" s="35"/>
       <c r="G4" t="s" s="5">
         <v>54</v>
       </c>
@@ -3763,6 +3875,15 @@
       <c r="N4" s="37">
         <v>9</v>
       </c>
+      <c r="O4" t="s" s="30">
+        <v>261</v>
+      </c>
+      <c r="P4" t="s" s="30">
+        <v>266</v>
+      </c>
+      <c r="R4" t="s" s="30">
+        <v>270</v>
+      </c>
     </row>
     <row r="5" ht="13.75" customHeight="1">
       <c r="A5" t="s" s="2">
@@ -3771,16 +3892,10 @@
       <c r="B5" t="s" s="2">
         <v>62</v>
       </c>
-      <c r="C5" t="s" s="33">
-        <v>51</v>
-      </c>
-      <c r="D5" t="s" s="33">
-        <v>52</v>
-      </c>
+      <c r="C5" s="33"/>
+      <c r="D5" s="33"/>
       <c r="E5" s="34"/>
-      <c r="F5" t="s" s="35">
-        <v>63</v>
-      </c>
+      <c r="F5" s="35"/>
       <c r="G5" t="s" s="5">
         <v>54</v>
       </c>
@@ -3801,6 +3916,15 @@
       <c r="N5" s="37">
         <v>9</v>
       </c>
+      <c r="O5" t="s" s="30">
+        <v>261</v>
+      </c>
+      <c r="P5" t="s" s="30">
+        <v>266</v>
+      </c>
+      <c r="R5" t="s" s="30">
+        <v>271</v>
+      </c>
     </row>
     <row r="6" ht="13.75" customHeight="1">
       <c r="A6" t="s" s="2">
@@ -3809,16 +3933,10 @@
       <c r="B6" t="s" s="2">
         <v>65</v>
       </c>
-      <c r="C6" t="s" s="33">
-        <v>51</v>
-      </c>
-      <c r="D6" t="s" s="33">
-        <v>52</v>
-      </c>
+      <c r="C6" s="33"/>
+      <c r="D6" s="33"/>
       <c r="E6" s="34"/>
-      <c r="F6" t="s" s="35">
-        <v>66</v>
-      </c>
+      <c r="F6" s="35"/>
       <c r="G6" t="s" s="5">
         <v>54</v>
       </c>
@@ -3839,6 +3957,15 @@
       <c r="N6" s="37">
         <v>9</v>
       </c>
+      <c r="O6" t="s" s="30">
+        <v>261</v>
+      </c>
+      <c r="P6" t="s" s="30">
+        <v>266</v>
+      </c>
+      <c r="R6" t="s" s="30">
+        <v>272</v>
+      </c>
     </row>
     <row r="7" ht="13.75" customHeight="1">
       <c r="A7" t="s" s="2">
@@ -3847,16 +3974,10 @@
       <c r="B7" t="s" s="2">
         <v>69</v>
       </c>
-      <c r="C7" t="s" s="33">
-        <v>51</v>
-      </c>
-      <c r="D7" t="s" s="33">
-        <v>52</v>
-      </c>
+      <c r="C7" s="33"/>
+      <c r="D7" s="33"/>
       <c r="E7" s="34"/>
-      <c r="F7" t="s" s="35">
-        <v>70</v>
-      </c>
+      <c r="F7" s="35"/>
       <c r="G7" t="s" s="5">
         <v>54</v>
       </c>
@@ -3877,6 +3998,15 @@
       <c r="N7" s="37">
         <v>9</v>
       </c>
+      <c r="O7" t="s" s="30">
+        <v>261</v>
+      </c>
+      <c r="P7" t="s" s="30">
+        <v>266</v>
+      </c>
+      <c r="R7" t="s" s="30">
+        <v>273</v>
+      </c>
     </row>
     <row r="8" ht="13.75" customHeight="1">
       <c r="A8" t="s" s="2">
@@ -3885,16 +4015,10 @@
       <c r="B8" t="s" s="2">
         <v>72</v>
       </c>
-      <c r="C8" t="s" s="33">
-        <v>51</v>
-      </c>
-      <c r="D8" t="s" s="33">
-        <v>52</v>
-      </c>
+      <c r="C8" s="33"/>
+      <c r="D8" s="33"/>
       <c r="E8" s="34"/>
-      <c r="F8" t="s" s="35">
-        <v>70</v>
-      </c>
+      <c r="F8" s="35"/>
       <c r="G8" t="s" s="5">
         <v>54</v>
       </c>
@@ -3915,6 +4039,15 @@
       <c r="N8" s="37">
         <v>9</v>
       </c>
+      <c r="O8" t="s" s="30">
+        <v>261</v>
+      </c>
+      <c r="P8" t="s" s="30">
+        <v>266</v>
+      </c>
+      <c r="R8" t="s" s="30">
+        <v>273</v>
+      </c>
     </row>
     <row r="9" ht="13.75" customHeight="1">
       <c r="A9" t="s" s="2">
@@ -3923,16 +4056,10 @@
       <c r="B9" t="s" s="2">
         <v>74</v>
       </c>
-      <c r="C9" t="s" s="33">
-        <v>51</v>
-      </c>
-      <c r="D9" t="s" s="33">
-        <v>52</v>
-      </c>
+      <c r="C9" s="33"/>
+      <c r="D9" s="33"/>
       <c r="E9" s="34"/>
-      <c r="F9" t="s" s="35">
-        <v>66</v>
-      </c>
+      <c r="F9" s="35"/>
       <c r="G9" t="s" s="5">
         <v>54</v>
       </c>
@@ -3953,6 +4080,15 @@
       <c r="N9" s="37">
         <v>9</v>
       </c>
+      <c r="O9" t="s" s="30">
+        <v>261</v>
+      </c>
+      <c r="P9" t="s" s="30">
+        <v>266</v>
+      </c>
+      <c r="R9" t="s" s="30">
+        <v>272</v>
+      </c>
     </row>
     <row r="10" ht="13.75" customHeight="1">
       <c r="A10" t="s" s="2">
@@ -3961,16 +4097,10 @@
       <c r="B10" t="s" s="2">
         <v>76</v>
       </c>
-      <c r="C10" t="s" s="33">
-        <v>51</v>
-      </c>
-      <c r="D10" t="s" s="33">
-        <v>52</v>
-      </c>
+      <c r="C10" s="33"/>
+      <c r="D10" s="33"/>
       <c r="E10" s="34"/>
-      <c r="F10" t="s" s="35">
-        <v>77</v>
-      </c>
+      <c r="F10" s="35"/>
       <c r="G10" t="s" s="5">
         <v>54</v>
       </c>
@@ -3991,6 +4121,15 @@
       <c r="N10" s="37">
         <v>9</v>
       </c>
+      <c r="O10" t="s" s="30">
+        <v>261</v>
+      </c>
+      <c r="P10" t="s" s="30">
+        <v>266</v>
+      </c>
+      <c r="R10" t="s" s="30">
+        <v>274</v>
+      </c>
     </row>
     <row r="11" ht="13.75" customHeight="1">
       <c r="A11" t="s" s="2">
@@ -3999,16 +4138,10 @@
       <c r="B11" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="C11" t="s" s="33">
-        <v>51</v>
-      </c>
-      <c r="D11" t="s" s="33">
-        <v>52</v>
-      </c>
+      <c r="C11" s="33"/>
+      <c r="D11" s="33"/>
       <c r="E11" s="34"/>
-      <c r="F11" t="s" s="35">
-        <v>66</v>
-      </c>
+      <c r="F11" s="35"/>
       <c r="G11" t="s" s="5">
         <v>54</v>
       </c>
@@ -4029,6 +4162,15 @@
       <c r="N11" s="37">
         <v>9</v>
       </c>
+      <c r="O11" t="s" s="30">
+        <v>261</v>
+      </c>
+      <c r="P11" t="s" s="30">
+        <v>266</v>
+      </c>
+      <c r="R11" t="s" s="30">
+        <v>272</v>
+      </c>
     </row>
     <row r="12" ht="13.75" customHeight="1">
       <c r="A12" t="s" s="2">
@@ -4037,16 +4179,10 @@
       <c r="B12" t="s" s="2">
         <v>81</v>
       </c>
-      <c r="C12" t="s" s="33">
-        <v>51</v>
-      </c>
-      <c r="D12" t="s" s="33">
-        <v>52</v>
-      </c>
+      <c r="C12" s="33"/>
+      <c r="D12" s="33"/>
       <c r="E12" s="34"/>
-      <c r="F12" t="s" s="35">
-        <v>53</v>
-      </c>
+      <c r="F12" s="35"/>
       <c r="G12" t="s" s="5">
         <v>54</v>
       </c>
@@ -4067,6 +4203,15 @@
       <c r="N12" s="37">
         <v>9</v>
       </c>
+      <c r="O12" t="s" s="30">
+        <v>261</v>
+      </c>
+      <c r="P12" t="s" s="30">
+        <v>266</v>
+      </c>
+      <c r="R12" t="s" s="30">
+        <v>270</v>
+      </c>
     </row>
     <row r="13" ht="13.75" customHeight="1">
       <c r="A13" t="s" s="2">
@@ -4075,16 +4220,10 @@
       <c r="B13" t="s" s="2">
         <v>83</v>
       </c>
-      <c r="C13" t="s" s="33">
-        <v>51</v>
-      </c>
-      <c r="D13" t="s" s="33">
-        <v>52</v>
-      </c>
+      <c r="C13" s="33"/>
+      <c r="D13" s="33"/>
       <c r="E13" s="34"/>
-      <c r="F13" t="s" s="35">
-        <v>66</v>
-      </c>
+      <c r="F13" s="35"/>
       <c r="G13" t="s" s="5">
         <v>54</v>
       </c>
@@ -4105,6 +4244,15 @@
       <c r="N13" s="37">
         <v>9</v>
       </c>
+      <c r="O13" t="s" s="30">
+        <v>261</v>
+      </c>
+      <c r="P13" t="s" s="30">
+        <v>266</v>
+      </c>
+      <c r="R13" t="s" s="30">
+        <v>272</v>
+      </c>
     </row>
     <row r="14" ht="13.75" customHeight="1">
       <c r="A14" t="s" s="2">
@@ -4113,16 +4261,10 @@
       <c r="B14" t="s" s="2">
         <v>85</v>
       </c>
-      <c r="C14" t="s" s="33">
-        <v>51</v>
-      </c>
-      <c r="D14" t="s" s="33">
-        <v>86</v>
-      </c>
+      <c r="C14" s="33"/>
+      <c r="D14" s="33"/>
       <c r="E14" s="34"/>
-      <c r="F14" t="s" s="35">
-        <v>87</v>
-      </c>
+      <c r="F14" s="35"/>
       <c r="G14" t="s" s="5">
         <v>54</v>
       </c>
@@ -4143,6 +4285,15 @@
       <c r="N14" s="37">
         <v>9</v>
       </c>
+      <c r="O14" t="s" s="30">
+        <v>261</v>
+      </c>
+      <c r="P14" t="s" s="30">
+        <v>267</v>
+      </c>
+      <c r="R14" t="s" s="30">
+        <v>275</v>
+      </c>
     </row>
     <row r="15" ht="13.75" customHeight="1">
       <c r="A15" t="s" s="2">
@@ -4151,16 +4302,10 @@
       <c r="B15" t="s" s="2">
         <v>89</v>
       </c>
-      <c r="C15" t="s" s="33">
-        <v>51</v>
-      </c>
-      <c r="D15" t="s" s="33">
-        <v>52</v>
-      </c>
+      <c r="C15" s="33"/>
+      <c r="D15" s="33"/>
       <c r="E15" s="34"/>
-      <c r="F15" t="s" s="35">
-        <v>90</v>
-      </c>
+      <c r="F15" s="35"/>
       <c r="G15" t="s" s="5">
         <v>54</v>
       </c>
@@ -4181,6 +4326,15 @@
       <c r="N15" s="37">
         <v>9</v>
       </c>
+      <c r="O15" t="s" s="30">
+        <v>261</v>
+      </c>
+      <c r="P15" t="s" s="30">
+        <v>266</v>
+      </c>
+      <c r="R15" t="s" s="30">
+        <v>276</v>
+      </c>
     </row>
     <row r="16" ht="13.75" customHeight="1">
       <c r="A16" t="s" s="2">
@@ -4189,16 +4343,10 @@
       <c r="B16" t="s" s="2">
         <v>92</v>
       </c>
-      <c r="C16" t="s" s="33">
-        <v>51</v>
-      </c>
-      <c r="D16" t="s" s="33">
-        <v>86</v>
-      </c>
+      <c r="C16" s="33"/>
+      <c r="D16" s="33"/>
       <c r="E16" s="34"/>
-      <c r="F16" t="s" s="35">
-        <v>87</v>
-      </c>
+      <c r="F16" s="35"/>
       <c r="G16" t="s" s="5">
         <v>54</v>
       </c>
@@ -4219,6 +4367,15 @@
       <c r="N16" s="37">
         <v>9</v>
       </c>
+      <c r="O16" t="s" s="30">
+        <v>261</v>
+      </c>
+      <c r="P16" t="s" s="30">
+        <v>267</v>
+      </c>
+      <c r="R16" t="s" s="30">
+        <v>275</v>
+      </c>
     </row>
     <row r="17" ht="13.75" customHeight="1">
       <c r="A17" t="s" s="2">
@@ -4227,16 +4384,10 @@
       <c r="B17" t="s" s="2">
         <v>94</v>
       </c>
-      <c r="C17" t="s" s="33">
-        <v>51</v>
-      </c>
-      <c r="D17" t="s" s="33">
-        <v>86</v>
-      </c>
+      <c r="C17" s="33"/>
+      <c r="D17" s="33"/>
       <c r="E17" s="34"/>
-      <c r="F17" t="s" s="35">
-        <v>87</v>
-      </c>
+      <c r="F17" s="35"/>
       <c r="G17" t="s" s="5">
         <v>54</v>
       </c>
@@ -4257,6 +4408,15 @@
       <c r="N17" s="37">
         <v>9</v>
       </c>
+      <c r="O17" t="s" s="30">
+        <v>261</v>
+      </c>
+      <c r="P17" t="s" s="30">
+        <v>267</v>
+      </c>
+      <c r="R17" t="s" s="30">
+        <v>275</v>
+      </c>
     </row>
     <row r="18" ht="13.75" customHeight="1">
       <c r="A18" t="s" s="2">
@@ -4265,16 +4425,10 @@
       <c r="B18" t="s" s="2">
         <v>96</v>
       </c>
-      <c r="C18" t="s" s="33">
-        <v>51</v>
-      </c>
-      <c r="D18" t="s" s="33">
-        <v>52</v>
-      </c>
+      <c r="C18" s="33"/>
+      <c r="D18" s="33"/>
       <c r="E18" s="34"/>
-      <c r="F18" t="s" s="35">
-        <v>63</v>
-      </c>
+      <c r="F18" s="35"/>
       <c r="G18" t="s" s="5">
         <v>54</v>
       </c>
@@ -4295,6 +4449,15 @@
       <c r="N18" s="37">
         <v>9</v>
       </c>
+      <c r="O18" t="s" s="30">
+        <v>261</v>
+      </c>
+      <c r="P18" t="s" s="30">
+        <v>266</v>
+      </c>
+      <c r="R18" t="s" s="30">
+        <v>271</v>
+      </c>
     </row>
     <row r="19" ht="13.75" customHeight="1">
       <c r="A19" t="s" s="2">
@@ -4303,16 +4466,10 @@
       <c r="B19" t="s" s="2">
         <v>98</v>
       </c>
-      <c r="C19" t="s" s="33">
-        <v>51</v>
-      </c>
-      <c r="D19" t="s" s="33">
-        <v>52</v>
-      </c>
+      <c r="C19" s="33"/>
+      <c r="D19" s="33"/>
       <c r="E19" s="34"/>
-      <c r="F19" t="s" s="35">
-        <v>63</v>
-      </c>
+      <c r="F19" s="35"/>
       <c r="G19" t="s" s="5">
         <v>54</v>
       </c>
@@ -4333,6 +4490,15 @@
       <c r="N19" s="37">
         <v>9</v>
       </c>
+      <c r="O19" t="s" s="30">
+        <v>261</v>
+      </c>
+      <c r="P19" t="s" s="30">
+        <v>266</v>
+      </c>
+      <c r="R19" t="s" s="30">
+        <v>271</v>
+      </c>
     </row>
     <row r="20" ht="13.75" customHeight="1">
       <c r="A20" t="s" s="2">
@@ -4341,16 +4507,10 @@
       <c r="B20" t="s" s="2">
         <v>100</v>
       </c>
-      <c r="C20" t="s" s="33">
-        <v>51</v>
-      </c>
-      <c r="D20" t="s" s="33">
-        <v>52</v>
-      </c>
+      <c r="C20" s="33"/>
+      <c r="D20" s="33"/>
       <c r="E20" s="34"/>
-      <c r="F20" t="s" s="35">
-        <v>101</v>
-      </c>
+      <c r="F20" s="35"/>
       <c r="G20" t="s" s="5">
         <v>54</v>
       </c>
@@ -4371,6 +4531,15 @@
       <c r="N20" s="37">
         <v>9</v>
       </c>
+      <c r="O20" t="s" s="30">
+        <v>261</v>
+      </c>
+      <c r="P20" t="s" s="30">
+        <v>266</v>
+      </c>
+      <c r="R20" t="s" s="30">
+        <v>277</v>
+      </c>
     </row>
     <row r="21" ht="13.75" customHeight="1">
       <c r="A21" t="s" s="2">
@@ -4379,16 +4548,10 @@
       <c r="B21" t="s" s="2">
         <v>103</v>
       </c>
-      <c r="C21" t="s" s="33">
-        <v>51</v>
-      </c>
-      <c r="D21" t="s" s="33">
-        <v>52</v>
-      </c>
+      <c r="C21" s="33"/>
+      <c r="D21" s="33"/>
       <c r="E21" s="34"/>
-      <c r="F21" t="s" s="35">
-        <v>90</v>
-      </c>
+      <c r="F21" s="35"/>
       <c r="G21" t="s" s="5">
         <v>54</v>
       </c>
@@ -4409,6 +4572,15 @@
       <c r="N21" s="37">
         <v>9</v>
       </c>
+      <c r="O21" t="s" s="30">
+        <v>261</v>
+      </c>
+      <c r="P21" t="s" s="30">
+        <v>266</v>
+      </c>
+      <c r="R21" t="s" s="30">
+        <v>276</v>
+      </c>
     </row>
     <row r="22" ht="13.75" customHeight="1">
       <c r="A22" t="s" s="2">
@@ -4417,16 +4589,10 @@
       <c r="B22" t="s" s="2">
         <v>105</v>
       </c>
-      <c r="C22" t="s" s="33">
-        <v>51</v>
-      </c>
-      <c r="D22" t="s" s="33">
-        <v>52</v>
-      </c>
+      <c r="C22" s="33"/>
+      <c r="D22" s="33"/>
       <c r="E22" s="34"/>
-      <c r="F22" t="s" s="35">
-        <v>70</v>
-      </c>
+      <c r="F22" s="35"/>
       <c r="G22" t="s" s="5">
         <v>54</v>
       </c>
@@ -4447,6 +4613,15 @@
       <c r="N22" s="37">
         <v>9</v>
       </c>
+      <c r="O22" t="s" s="30">
+        <v>261</v>
+      </c>
+      <c r="P22" t="s" s="30">
+        <v>266</v>
+      </c>
+      <c r="R22" t="s" s="30">
+        <v>273</v>
+      </c>
     </row>
     <row r="23" ht="13.75" customHeight="1">
       <c r="A23" t="s" s="2">
@@ -4455,16 +4630,10 @@
       <c r="B23" t="s" s="2">
         <v>107</v>
       </c>
-      <c r="C23" t="s" s="33">
-        <v>51</v>
-      </c>
-      <c r="D23" t="s" s="33">
-        <v>52</v>
-      </c>
+      <c r="C23" s="33"/>
+      <c r="D23" s="33"/>
       <c r="E23" s="34"/>
-      <c r="F23" t="s" s="35">
-        <v>108</v>
-      </c>
+      <c r="F23" s="35"/>
       <c r="G23" t="s" s="5">
         <v>54</v>
       </c>
@@ -4485,6 +4654,15 @@
       <c r="N23" s="37">
         <v>9</v>
       </c>
+      <c r="O23" t="s" s="30">
+        <v>261</v>
+      </c>
+      <c r="P23" t="s" s="30">
+        <v>266</v>
+      </c>
+      <c r="R23" t="s" s="30">
+        <v>278</v>
+      </c>
     </row>
     <row r="24" ht="13.75" customHeight="1">
       <c r="A24" t="s" s="2">
@@ -4493,16 +4671,10 @@
       <c r="B24" t="s" s="2">
         <v>110</v>
       </c>
-      <c r="C24" t="s" s="33">
-        <v>51</v>
-      </c>
-      <c r="D24" t="s" s="33">
-        <v>86</v>
-      </c>
+      <c r="C24" s="33"/>
+      <c r="D24" s="33"/>
       <c r="E24" s="34"/>
-      <c r="F24" t="s" s="35">
-        <v>87</v>
-      </c>
+      <c r="F24" s="35"/>
       <c r="G24" t="s" s="5">
         <v>54</v>
       </c>
@@ -4523,6 +4695,15 @@
       <c r="N24" s="37">
         <v>9</v>
       </c>
+      <c r="O24" t="s" s="30">
+        <v>261</v>
+      </c>
+      <c r="P24" t="s" s="30">
+        <v>267</v>
+      </c>
+      <c r="R24" t="s" s="30">
+        <v>275</v>
+      </c>
     </row>
     <row r="25" ht="13.75" customHeight="1">
       <c r="A25" t="s" s="2">
@@ -4531,16 +4712,10 @@
       <c r="B25" t="s" s="2">
         <v>112</v>
       </c>
-      <c r="C25" t="s" s="33">
-        <v>51</v>
-      </c>
-      <c r="D25" t="s" s="33">
-        <v>52</v>
-      </c>
+      <c r="C25" s="33"/>
+      <c r="D25" s="33"/>
       <c r="E25" s="34"/>
-      <c r="F25" t="s" s="35">
-        <v>87</v>
-      </c>
+      <c r="F25" s="35"/>
       <c r="G25" t="s" s="5">
         <v>54</v>
       </c>
@@ -4561,6 +4736,15 @@
       <c r="N25" s="37">
         <v>9</v>
       </c>
+      <c r="O25" t="s" s="30">
+        <v>261</v>
+      </c>
+      <c r="P25" t="s" s="30">
+        <v>266</v>
+      </c>
+      <c r="R25" t="s" s="30">
+        <v>275</v>
+      </c>
     </row>
     <row r="26" ht="13.75" customHeight="1">
       <c r="A26" t="s" s="2">
@@ -4569,16 +4753,10 @@
       <c r="B26" t="s" s="2">
         <v>114</v>
       </c>
-      <c r="C26" t="s" s="33">
-        <v>51</v>
-      </c>
-      <c r="D26" t="s" s="33">
-        <v>52</v>
-      </c>
+      <c r="C26" s="33"/>
+      <c r="D26" s="33"/>
       <c r="E26" s="34"/>
-      <c r="F26" t="s" s="35">
-        <v>77</v>
-      </c>
+      <c r="F26" s="35"/>
       <c r="G26" t="s" s="5">
         <v>54</v>
       </c>
@@ -4599,6 +4777,15 @@
       <c r="N26" s="37">
         <v>9</v>
       </c>
+      <c r="O26" t="s" s="30">
+        <v>261</v>
+      </c>
+      <c r="P26" t="s" s="30">
+        <v>266</v>
+      </c>
+      <c r="R26" t="s" s="30">
+        <v>274</v>
+      </c>
     </row>
     <row r="27" ht="13.75" customHeight="1">
       <c r="A27" t="s" s="2">
@@ -4607,16 +4794,10 @@
       <c r="B27" t="s" s="2">
         <v>116</v>
       </c>
-      <c r="C27" t="s" s="33">
-        <v>51</v>
-      </c>
-      <c r="D27" t="s" s="33">
-        <v>52</v>
-      </c>
+      <c r="C27" s="33"/>
+      <c r="D27" s="33"/>
       <c r="E27" s="34"/>
-      <c r="F27" t="s" s="35">
-        <v>108</v>
-      </c>
+      <c r="F27" s="35"/>
       <c r="G27" t="s" s="5">
         <v>54</v>
       </c>
@@ -4637,6 +4818,15 @@
       <c r="N27" s="37">
         <v>9</v>
       </c>
+      <c r="O27" t="s" s="30">
+        <v>261</v>
+      </c>
+      <c r="P27" t="s" s="30">
+        <v>266</v>
+      </c>
+      <c r="R27" t="s" s="30">
+        <v>278</v>
+      </c>
     </row>
     <row r="28" ht="13.75" customHeight="1">
       <c r="A28" t="s" s="2">
@@ -4645,16 +4835,10 @@
       <c r="B28" t="s" s="2">
         <v>118</v>
       </c>
-      <c r="C28" t="s" s="33">
-        <v>51</v>
-      </c>
-      <c r="D28" t="s" s="33">
-        <v>52</v>
-      </c>
+      <c r="C28" s="33"/>
+      <c r="D28" s="33"/>
       <c r="E28" s="34"/>
-      <c r="F28" t="s" s="35">
-        <v>63</v>
-      </c>
+      <c r="F28" s="35"/>
       <c r="G28" t="s" s="5">
         <v>54</v>
       </c>
@@ -4675,6 +4859,15 @@
       <c r="N28" s="37">
         <v>9</v>
       </c>
+      <c r="O28" t="s" s="30">
+        <v>261</v>
+      </c>
+      <c r="P28" t="s" s="30">
+        <v>266</v>
+      </c>
+      <c r="R28" t="s" s="30">
+        <v>271</v>
+      </c>
     </row>
     <row r="29" ht="13.75" customHeight="1">
       <c r="A29" t="s" s="2">
@@ -4683,16 +4876,10 @@
       <c r="B29" t="s" s="2">
         <v>120</v>
       </c>
-      <c r="C29" t="s" s="33">
-        <v>51</v>
-      </c>
-      <c r="D29" t="s" s="33">
-        <v>86</v>
-      </c>
+      <c r="C29" s="33"/>
+      <c r="D29" s="33"/>
       <c r="E29" s="34"/>
-      <c r="F29" t="s" s="35">
-        <v>87</v>
-      </c>
+      <c r="F29" s="35"/>
       <c r="G29" t="s" s="5">
         <v>54</v>
       </c>
@@ -4713,6 +4900,15 @@
       <c r="N29" s="37">
         <v>3</v>
       </c>
+      <c r="O29" t="s" s="30">
+        <v>261</v>
+      </c>
+      <c r="P29" t="s" s="30">
+        <v>267</v>
+      </c>
+      <c r="R29" t="s" s="30">
+        <v>275</v>
+      </c>
     </row>
     <row r="30" ht="13.75" customHeight="1">
       <c r="A30" t="s" s="2">
@@ -4721,16 +4917,10 @@
       <c r="B30" t="s" s="2">
         <v>122</v>
       </c>
-      <c r="C30" t="s" s="33">
-        <v>51</v>
-      </c>
-      <c r="D30" t="s" s="33">
-        <v>52</v>
-      </c>
+      <c r="C30" s="33"/>
+      <c r="D30" s="33"/>
       <c r="E30" s="34"/>
-      <c r="F30" t="s" s="35">
-        <v>108</v>
-      </c>
+      <c r="F30" s="35"/>
       <c r="G30" t="s" s="5">
         <v>54</v>
       </c>
@@ -4751,6 +4941,15 @@
       <c r="N30" s="37">
         <v>9</v>
       </c>
+      <c r="O30" t="s" s="30">
+        <v>261</v>
+      </c>
+      <c r="P30" t="s" s="30">
+        <v>266</v>
+      </c>
+      <c r="R30" t="s" s="30">
+        <v>278</v>
+      </c>
     </row>
     <row r="31" ht="13.75" customHeight="1">
       <c r="A31" t="s" s="2">
@@ -4759,16 +4958,10 @@
       <c r="B31" t="s" s="2">
         <v>124</v>
       </c>
-      <c r="C31" t="s" s="33">
-        <v>51</v>
-      </c>
-      <c r="D31" t="s" s="33">
-        <v>52</v>
-      </c>
+      <c r="C31" s="33"/>
+      <c r="D31" s="33"/>
       <c r="E31" s="34"/>
-      <c r="F31" t="s" s="35">
-        <v>108</v>
-      </c>
+      <c r="F31" s="35"/>
       <c r="G31" t="s" s="5">
         <v>54</v>
       </c>
@@ -4789,6 +4982,15 @@
       <c r="N31" s="37">
         <v>9</v>
       </c>
+      <c r="O31" t="s" s="30">
+        <v>261</v>
+      </c>
+      <c r="P31" t="s" s="30">
+        <v>266</v>
+      </c>
+      <c r="R31" t="s" s="30">
+        <v>278</v>
+      </c>
     </row>
     <row r="32" ht="13.75" customHeight="1">
       <c r="A32" t="s" s="2">
@@ -4797,16 +4999,10 @@
       <c r="B32" t="s" s="2">
         <v>126</v>
       </c>
-      <c r="C32" t="s" s="33">
-        <v>51</v>
-      </c>
-      <c r="D32" t="s" s="33">
-        <v>52</v>
-      </c>
+      <c r="C32" s="33"/>
+      <c r="D32" s="33"/>
       <c r="E32" s="34"/>
-      <c r="F32" t="s" s="35">
-        <v>108</v>
-      </c>
+      <c r="F32" s="35"/>
       <c r="G32" t="s" s="5">
         <v>54</v>
       </c>
@@ -4827,6 +5023,15 @@
       <c r="N32" s="37">
         <v>9</v>
       </c>
+      <c r="O32" t="s" s="30">
+        <v>261</v>
+      </c>
+      <c r="P32" t="s" s="30">
+        <v>266</v>
+      </c>
+      <c r="R32" t="s" s="30">
+        <v>278</v>
+      </c>
     </row>
     <row r="33" ht="13.75" customHeight="1">
       <c r="A33" t="s" s="2">
@@ -4835,16 +5040,10 @@
       <c r="B33" t="s" s="2">
         <v>128</v>
       </c>
-      <c r="C33" t="s" s="33">
-        <v>51</v>
-      </c>
-      <c r="D33" t="s" s="33">
-        <v>52</v>
-      </c>
+      <c r="C33" s="33"/>
+      <c r="D33" s="33"/>
       <c r="E33" s="34"/>
-      <c r="F33" t="s" s="35">
-        <v>87</v>
-      </c>
+      <c r="F33" s="35"/>
       <c r="G33" t="s" s="5">
         <v>54</v>
       </c>
@@ -4865,6 +5064,15 @@
       <c r="N33" s="37">
         <v>9</v>
       </c>
+      <c r="O33" t="s" s="30">
+        <v>261</v>
+      </c>
+      <c r="P33" t="s" s="30">
+        <v>266</v>
+      </c>
+      <c r="R33" t="s" s="30">
+        <v>275</v>
+      </c>
     </row>
     <row r="34" ht="13.75" customHeight="1">
       <c r="A34" t="s" s="2">
@@ -4873,16 +5081,10 @@
       <c r="B34" t="s" s="2">
         <v>130</v>
       </c>
-      <c r="C34" t="s" s="33">
-        <v>51</v>
-      </c>
-      <c r="D34" t="s" s="33">
-        <v>52</v>
-      </c>
+      <c r="C34" s="33"/>
+      <c r="D34" s="33"/>
       <c r="E34" s="34"/>
-      <c r="F34" t="s" s="35">
-        <v>131</v>
-      </c>
+      <c r="F34" s="35"/>
       <c r="G34" t="s" s="5">
         <v>54</v>
       </c>
@@ -4903,6 +5105,15 @@
       <c r="N34" s="37">
         <v>9</v>
       </c>
+      <c r="O34" t="s" s="30">
+        <v>261</v>
+      </c>
+      <c r="P34" t="s" s="30">
+        <v>266</v>
+      </c>
+      <c r="R34" t="s" s="30">
+        <v>279</v>
+      </c>
     </row>
     <row r="35" ht="13.75" customHeight="1">
       <c r="A35" t="s" s="2">
@@ -4911,16 +5122,10 @@
       <c r="B35" t="s" s="2">
         <v>133</v>
       </c>
-      <c r="C35" t="s" s="33">
-        <v>51</v>
-      </c>
-      <c r="D35" t="s" s="33">
-        <v>52</v>
-      </c>
+      <c r="C35" s="33"/>
+      <c r="D35" s="33"/>
       <c r="E35" s="34"/>
-      <c r="F35" t="s" s="35">
-        <v>108</v>
-      </c>
+      <c r="F35" s="35"/>
       <c r="G35" t="s" s="5">
         <v>54</v>
       </c>
@@ -4941,6 +5146,15 @@
       <c r="N35" s="37">
         <v>9</v>
       </c>
+      <c r="O35" t="s" s="30">
+        <v>261</v>
+      </c>
+      <c r="P35" t="s" s="30">
+        <v>266</v>
+      </c>
+      <c r="R35" t="s" s="30">
+        <v>278</v>
+      </c>
     </row>
     <row r="36" ht="13.75" customHeight="1">
       <c r="A36" t="s" s="2">
@@ -4949,16 +5163,10 @@
       <c r="B36" t="s" s="2">
         <v>135</v>
       </c>
-      <c r="C36" t="s" s="33">
-        <v>51</v>
-      </c>
-      <c r="D36" t="s" s="33">
-        <v>52</v>
-      </c>
+      <c r="C36" s="33"/>
+      <c r="D36" s="33"/>
       <c r="E36" s="34"/>
-      <c r="F36" t="s" s="35">
-        <v>131</v>
-      </c>
+      <c r="F36" s="35"/>
       <c r="G36" t="s" s="5">
         <v>54</v>
       </c>
@@ -4979,6 +5187,15 @@
       <c r="N36" s="37">
         <v>9</v>
       </c>
+      <c r="O36" t="s" s="30">
+        <v>261</v>
+      </c>
+      <c r="P36" t="s" s="30">
+        <v>266</v>
+      </c>
+      <c r="R36" t="s" s="30">
+        <v>279</v>
+      </c>
     </row>
     <row r="37" ht="13.75" customHeight="1">
       <c r="A37" t="s" s="2">
@@ -4987,16 +5204,10 @@
       <c r="B37" t="s" s="2">
         <v>137</v>
       </c>
-      <c r="C37" t="s" s="33">
-        <v>51</v>
-      </c>
-      <c r="D37" t="s" s="33">
-        <v>52</v>
-      </c>
+      <c r="C37" s="33"/>
+      <c r="D37" s="33"/>
       <c r="E37" s="34"/>
-      <c r="F37" t="s" s="35">
-        <v>108</v>
-      </c>
+      <c r="F37" s="35"/>
       <c r="G37" t="s" s="5">
         <v>54</v>
       </c>
@@ -5017,6 +5228,15 @@
       <c r="N37" s="37">
         <v>9</v>
       </c>
+      <c r="O37" t="s" s="30">
+        <v>261</v>
+      </c>
+      <c r="P37" t="s" s="30">
+        <v>266</v>
+      </c>
+      <c r="R37" t="s" s="30">
+        <v>278</v>
+      </c>
     </row>
     <row r="38" ht="13.75" customHeight="1">
       <c r="A38" t="s" s="2">
@@ -5025,16 +5245,10 @@
       <c r="B38" t="s" s="2">
         <v>139</v>
       </c>
-      <c r="C38" t="s" s="33">
-        <v>51</v>
-      </c>
-      <c r="D38" t="s" s="33">
-        <v>52</v>
-      </c>
+      <c r="C38" s="33"/>
+      <c r="D38" s="33"/>
       <c r="E38" s="34"/>
-      <c r="F38" t="s" s="35">
-        <v>108</v>
-      </c>
+      <c r="F38" s="35"/>
       <c r="G38" t="s" s="5">
         <v>54</v>
       </c>
@@ -5055,6 +5269,15 @@
       <c r="N38" s="37">
         <v>9</v>
       </c>
+      <c r="O38" t="s" s="30">
+        <v>261</v>
+      </c>
+      <c r="P38" t="s" s="30">
+        <v>266</v>
+      </c>
+      <c r="R38" t="s" s="30">
+        <v>278</v>
+      </c>
     </row>
     <row r="39" ht="13.75" customHeight="1">
       <c r="A39" t="s" s="2">
@@ -5063,16 +5286,10 @@
       <c r="B39" t="s" s="2">
         <v>141</v>
       </c>
-      <c r="C39" t="s" s="33">
-        <v>51</v>
-      </c>
-      <c r="D39" t="s" s="33">
-        <v>52</v>
-      </c>
+      <c r="C39" s="33"/>
+      <c r="D39" s="33"/>
       <c r="E39" s="34"/>
-      <c r="F39" t="s" s="35">
-        <v>131</v>
-      </c>
+      <c r="F39" s="35"/>
       <c r="G39" t="s" s="5">
         <v>54</v>
       </c>
@@ -5093,6 +5310,15 @@
       <c r="N39" s="37">
         <v>9</v>
       </c>
+      <c r="O39" t="s" s="30">
+        <v>261</v>
+      </c>
+      <c r="P39" t="s" s="30">
+        <v>266</v>
+      </c>
+      <c r="R39" t="s" s="30">
+        <v>279</v>
+      </c>
     </row>
     <row r="40" ht="13.75" customHeight="1">
       <c r="A40" t="s" s="2">
@@ -5101,16 +5327,10 @@
       <c r="B40" t="s" s="2">
         <v>143</v>
       </c>
-      <c r="C40" t="s" s="33">
-        <v>51</v>
-      </c>
-      <c r="D40" t="s" s="33">
-        <v>52</v>
-      </c>
+      <c r="C40" s="33"/>
+      <c r="D40" s="33"/>
       <c r="E40" s="34"/>
-      <c r="F40" t="s" s="35">
-        <v>108</v>
-      </c>
+      <c r="F40" s="35"/>
       <c r="G40" t="s" s="5">
         <v>54</v>
       </c>
@@ -5131,6 +5351,15 @@
       <c r="N40" s="37">
         <v>9</v>
       </c>
+      <c r="O40" t="s" s="30">
+        <v>261</v>
+      </c>
+      <c r="P40" t="s" s="30">
+        <v>266</v>
+      </c>
+      <c r="R40" t="s" s="30">
+        <v>278</v>
+      </c>
     </row>
     <row r="41" ht="13.75" customHeight="1">
       <c r="A41" t="s" s="2">
@@ -5139,16 +5368,10 @@
       <c r="B41" t="s" s="2">
         <v>145</v>
       </c>
-      <c r="C41" t="s" s="33">
-        <v>51</v>
-      </c>
-      <c r="D41" t="s" s="33">
-        <v>52</v>
-      </c>
+      <c r="C41" s="33"/>
+      <c r="D41" s="33"/>
       <c r="E41" s="34"/>
-      <c r="F41" t="s" s="35">
-        <v>90</v>
-      </c>
+      <c r="F41" s="35"/>
       <c r="G41" t="s" s="5">
         <v>54</v>
       </c>
@@ -5169,6 +5392,15 @@
       <c r="N41" s="37">
         <v>9</v>
       </c>
+      <c r="O41" t="s" s="30">
+        <v>261</v>
+      </c>
+      <c r="P41" t="s" s="30">
+        <v>266</v>
+      </c>
+      <c r="R41" t="s" s="30">
+        <v>276</v>
+      </c>
     </row>
     <row r="42" ht="13.75" customHeight="1">
       <c r="A42" t="s" s="2">
@@ -5177,16 +5409,10 @@
       <c r="B42" t="s" s="2">
         <v>147</v>
       </c>
-      <c r="C42" t="s" s="33">
-        <v>51</v>
-      </c>
-      <c r="D42" t="s" s="33">
-        <v>52</v>
-      </c>
+      <c r="C42" s="33"/>
+      <c r="D42" s="33"/>
       <c r="E42" s="34"/>
-      <c r="F42" t="s" s="35">
-        <v>108</v>
-      </c>
+      <c r="F42" s="35"/>
       <c r="G42" t="s" s="5">
         <v>54</v>
       </c>
@@ -5207,6 +5433,15 @@
       <c r="N42" s="37">
         <v>9</v>
       </c>
+      <c r="O42" t="s" s="30">
+        <v>261</v>
+      </c>
+      <c r="P42" t="s" s="30">
+        <v>266</v>
+      </c>
+      <c r="R42" t="s" s="30">
+        <v>278</v>
+      </c>
     </row>
     <row r="43" ht="13.75" customHeight="1">
       <c r="A43" t="s" s="2">
@@ -5215,16 +5450,10 @@
       <c r="B43" t="s" s="2">
         <v>149</v>
       </c>
-      <c r="C43" t="s" s="33">
-        <v>51</v>
-      </c>
-      <c r="D43" t="s" s="33">
-        <v>52</v>
-      </c>
+      <c r="C43" s="33"/>
+      <c r="D43" s="33"/>
       <c r="E43" s="34"/>
-      <c r="F43" t="s" s="35">
-        <v>66</v>
-      </c>
+      <c r="F43" s="35"/>
       <c r="G43" t="s" s="5">
         <v>54</v>
       </c>
@@ -5245,6 +5474,15 @@
       <c r="N43" s="37">
         <v>9</v>
       </c>
+      <c r="O43" t="s" s="30">
+        <v>261</v>
+      </c>
+      <c r="P43" t="s" s="30">
+        <v>266</v>
+      </c>
+      <c r="R43" t="s" s="30">
+        <v>272</v>
+      </c>
     </row>
     <row r="44" ht="13.75" customHeight="1">
       <c r="A44" t="s" s="2">
@@ -5253,16 +5491,10 @@
       <c r="B44" t="s" s="2">
         <v>151</v>
       </c>
-      <c r="C44" t="s" s="33">
-        <v>51</v>
-      </c>
-      <c r="D44" t="s" s="33">
-        <v>52</v>
-      </c>
+      <c r="C44" s="33"/>
+      <c r="D44" s="33"/>
       <c r="E44" s="34"/>
-      <c r="F44" t="s" s="35">
-        <v>70</v>
-      </c>
+      <c r="F44" s="35"/>
       <c r="G44" t="s" s="5">
         <v>54</v>
       </c>
@@ -5283,6 +5515,15 @@
       <c r="N44" s="37">
         <v>3</v>
       </c>
+      <c r="O44" t="s" s="30">
+        <v>261</v>
+      </c>
+      <c r="P44" t="s" s="30">
+        <v>266</v>
+      </c>
+      <c r="R44" t="s" s="30">
+        <v>273</v>
+      </c>
     </row>
     <row r="45" ht="13.75" customHeight="1">
       <c r="A45" t="s" s="2">
@@ -5291,16 +5532,10 @@
       <c r="B45" t="s" s="2">
         <v>153</v>
       </c>
-      <c r="C45" t="s" s="33">
-        <v>51</v>
-      </c>
-      <c r="D45" t="s" s="33">
-        <v>52</v>
-      </c>
+      <c r="C45" s="33"/>
+      <c r="D45" s="33"/>
       <c r="E45" s="34"/>
-      <c r="F45" t="s" s="35">
-        <v>108</v>
-      </c>
+      <c r="F45" s="35"/>
       <c r="G45" t="s" s="5">
         <v>54</v>
       </c>
@@ -5321,6 +5556,15 @@
       <c r="N45" s="37">
         <v>9</v>
       </c>
+      <c r="O45" t="s" s="30">
+        <v>261</v>
+      </c>
+      <c r="P45" t="s" s="30">
+        <v>266</v>
+      </c>
+      <c r="R45" t="s" s="30">
+        <v>278</v>
+      </c>
     </row>
     <row r="46" ht="13.75" customHeight="1">
       <c r="A46" t="s" s="2">
@@ -5329,16 +5573,10 @@
       <c r="B46" t="s" s="2">
         <v>155</v>
       </c>
-      <c r="C46" t="s" s="33">
-        <v>51</v>
-      </c>
-      <c r="D46" t="s" s="33">
-        <v>52</v>
-      </c>
+      <c r="C46" s="33"/>
+      <c r="D46" s="33"/>
       <c r="E46" s="34"/>
-      <c r="F46" t="s" s="35">
-        <v>108</v>
-      </c>
+      <c r="F46" s="35"/>
       <c r="G46" t="s" s="5">
         <v>54</v>
       </c>
@@ -5359,6 +5597,15 @@
       <c r="N46" s="37">
         <v>6</v>
       </c>
+      <c r="O46" t="s" s="30">
+        <v>261</v>
+      </c>
+      <c r="P46" t="s" s="30">
+        <v>266</v>
+      </c>
+      <c r="R46" t="s" s="30">
+        <v>278</v>
+      </c>
     </row>
     <row r="47" ht="13.75" customHeight="1">
       <c r="A47" t="s" s="2">
@@ -5367,16 +5614,10 @@
       <c r="B47" t="s" s="2">
         <v>157</v>
       </c>
-      <c r="C47" t="s" s="33">
-        <v>51</v>
-      </c>
-      <c r="D47" t="s" s="33">
-        <v>86</v>
-      </c>
+      <c r="C47" s="33"/>
+      <c r="D47" s="33"/>
       <c r="E47" s="34"/>
-      <c r="F47" t="s" s="35">
-        <v>87</v>
-      </c>
+      <c r="F47" s="35"/>
       <c r="G47" t="s" s="5">
         <v>54</v>
       </c>
@@ -5397,6 +5638,15 @@
       <c r="N47" s="37">
         <v>6</v>
       </c>
+      <c r="O47" t="s" s="30">
+        <v>261</v>
+      </c>
+      <c r="P47" t="s" s="30">
+        <v>267</v>
+      </c>
+      <c r="R47" t="s" s="30">
+        <v>275</v>
+      </c>
     </row>
     <row r="48" ht="13.75" customHeight="1">
       <c r="A48" t="s" s="38">
@@ -5405,16 +5655,10 @@
       <c r="B48" t="s" s="38">
         <v>159</v>
       </c>
-      <c r="C48" t="s" s="39">
-        <v>51</v>
-      </c>
-      <c r="D48" t="s" s="33">
-        <v>52</v>
-      </c>
+      <c r="C48" s="39"/>
+      <c r="D48" s="33"/>
       <c r="E48" s="34"/>
-      <c r="F48" t="s" s="35">
-        <v>90</v>
-      </c>
+      <c r="F48" s="35"/>
       <c r="G48" t="s" s="5">
         <v>54</v>
       </c>
@@ -5435,15 +5679,22 @@
       <c r="N48" s="37">
         <v>8</v>
       </c>
+      <c r="O48" t="s" s="30">
+        <v>261</v>
+      </c>
+      <c r="P48" t="s" s="30">
+        <v>266</v>
+      </c>
+      <c r="R48" t="s" s="30">
+        <v>276</v>
+      </c>
     </row>
     <row r="49" ht="14.7" customHeight="1">
       <c r="A49" t="s" s="40">
         <v>160</v>
       </c>
       <c r="B49" s="41"/>
-      <c r="C49" t="s" s="42">
-        <v>161</v>
-      </c>
+      <c r="C49" s="42"/>
       <c r="D49" s="43"/>
       <c r="E49" s="6"/>
       <c r="F49" s="44"/>
@@ -5463,15 +5714,16 @@
         <v>56</v>
       </c>
       <c r="N49" s="7"/>
+      <c r="O49" t="s" s="30">
+        <v>262</v>
+      </c>
     </row>
     <row r="50" ht="14.7" customHeight="1">
       <c r="A50" t="s" s="40">
         <v>162</v>
       </c>
       <c r="B50" s="41"/>
-      <c r="C50" t="s" s="42">
-        <v>161</v>
-      </c>
+      <c r="C50" s="42"/>
       <c r="D50" s="43"/>
       <c r="E50" s="6"/>
       <c r="F50" s="6"/>
@@ -5491,15 +5743,16 @@
         <v>56</v>
       </c>
       <c r="N50" s="7"/>
+      <c r="O50" t="s" s="30">
+        <v>262</v>
+      </c>
     </row>
     <row r="51" ht="14.7" customHeight="1">
       <c r="A51" t="s" s="40">
         <v>163</v>
       </c>
       <c r="B51" s="41"/>
-      <c r="C51" t="s" s="42">
-        <v>161</v>
-      </c>
+      <c r="C51" s="42"/>
       <c r="D51" s="43"/>
       <c r="E51" s="6"/>
       <c r="F51" s="6"/>
@@ -5519,15 +5772,16 @@
         <v>56</v>
       </c>
       <c r="N51" s="7"/>
+      <c r="O51" t="s" s="30">
+        <v>262</v>
+      </c>
     </row>
     <row r="52" ht="14.7" customHeight="1">
       <c r="A52" t="s" s="40">
         <v>164</v>
       </c>
       <c r="B52" s="41"/>
-      <c r="C52" t="s" s="42">
-        <v>161</v>
-      </c>
+      <c r="C52" s="42"/>
       <c r="D52" s="43"/>
       <c r="E52" s="6"/>
       <c r="F52" s="6"/>
@@ -5547,15 +5801,16 @@
         <v>56</v>
       </c>
       <c r="N52" s="7"/>
+      <c r="O52" t="s" s="30">
+        <v>262</v>
+      </c>
     </row>
     <row r="53" ht="14.7" customHeight="1">
       <c r="A53" t="s" s="40">
         <v>165</v>
       </c>
       <c r="B53" s="41"/>
-      <c r="C53" t="s" s="42">
-        <v>161</v>
-      </c>
+      <c r="C53" s="42"/>
       <c r="D53" s="43"/>
       <c r="E53" s="6"/>
       <c r="F53" s="6"/>
@@ -5575,15 +5830,16 @@
         <v>56</v>
       </c>
       <c r="N53" s="7"/>
+      <c r="O53" t="s" s="30">
+        <v>262</v>
+      </c>
     </row>
     <row r="54" ht="14.7" customHeight="1">
       <c r="A54" t="s" s="40">
         <v>166</v>
       </c>
       <c r="B54" s="41"/>
-      <c r="C54" t="s" s="42">
-        <v>161</v>
-      </c>
+      <c r="C54" s="42"/>
       <c r="D54" s="43"/>
       <c r="E54" s="6"/>
       <c r="F54" s="6"/>
@@ -5603,15 +5859,16 @@
         <v>56</v>
       </c>
       <c r="N54" s="7"/>
+      <c r="O54" t="s" s="30">
+        <v>262</v>
+      </c>
     </row>
     <row r="55" ht="14.7" customHeight="1">
       <c r="A55" t="s" s="40">
         <v>167</v>
       </c>
       <c r="B55" s="41"/>
-      <c r="C55" t="s" s="42">
-        <v>161</v>
-      </c>
+      <c r="C55" s="42"/>
       <c r="D55" s="43"/>
       <c r="E55" s="6"/>
       <c r="F55" s="6"/>
@@ -5631,15 +5888,16 @@
         <v>56</v>
       </c>
       <c r="N55" s="7"/>
+      <c r="O55" t="s" s="30">
+        <v>262</v>
+      </c>
     </row>
     <row r="56" ht="14.7" customHeight="1">
       <c r="A56" t="s" s="40">
         <v>168</v>
       </c>
       <c r="B56" s="41"/>
-      <c r="C56" t="s" s="42">
-        <v>161</v>
-      </c>
+      <c r="C56" s="42"/>
       <c r="D56" s="43"/>
       <c r="E56" s="6"/>
       <c r="F56" s="6"/>
@@ -5659,15 +5917,16 @@
         <v>56</v>
       </c>
       <c r="N56" s="7"/>
+      <c r="O56" t="s" s="30">
+        <v>262</v>
+      </c>
     </row>
     <row r="57" ht="14.7" customHeight="1">
       <c r="A57" t="s" s="40">
         <v>169</v>
       </c>
       <c r="B57" s="41"/>
-      <c r="C57" t="s" s="42">
-        <v>161</v>
-      </c>
+      <c r="C57" s="42"/>
       <c r="D57" s="43"/>
       <c r="E57" s="6"/>
       <c r="F57" s="6"/>
@@ -5687,15 +5946,16 @@
         <v>56</v>
       </c>
       <c r="N57" s="7"/>
+      <c r="O57" t="s" s="30">
+        <v>262</v>
+      </c>
     </row>
     <row r="58" ht="14.7" customHeight="1">
       <c r="A58" t="s" s="40">
         <v>170</v>
       </c>
       <c r="B58" s="41"/>
-      <c r="C58" t="s" s="42">
-        <v>161</v>
-      </c>
+      <c r="C58" s="42"/>
       <c r="D58" s="43"/>
       <c r="E58" s="6"/>
       <c r="F58" s="6"/>
@@ -5715,15 +5975,16 @@
         <v>56</v>
       </c>
       <c r="N58" s="7"/>
+      <c r="O58" t="s" s="30">
+        <v>262</v>
+      </c>
     </row>
     <row r="59" ht="13.65" customHeight="1">
       <c r="A59" t="s" s="40">
         <v>171</v>
       </c>
       <c r="B59" s="41"/>
-      <c r="C59" t="s" s="42">
-        <v>161</v>
-      </c>
+      <c r="C59" s="42"/>
       <c r="D59" s="43"/>
       <c r="E59" s="6"/>
       <c r="F59" s="6"/>
@@ -5743,15 +6004,16 @@
         <v>56</v>
       </c>
       <c r="N59" s="7"/>
+      <c r="O59" t="s" s="30">
+        <v>262</v>
+      </c>
     </row>
     <row r="60" ht="13.65" customHeight="1">
       <c r="A60" t="s" s="40">
         <v>172</v>
       </c>
       <c r="B60" s="41"/>
-      <c r="C60" t="s" s="42">
-        <v>161</v>
-      </c>
+      <c r="C60" s="42"/>
       <c r="D60" s="43"/>
       <c r="E60" s="6"/>
       <c r="F60" s="6"/>
@@ -5771,15 +6033,16 @@
         <v>56</v>
       </c>
       <c r="N60" s="7"/>
+      <c r="O60" t="s" s="30">
+        <v>262</v>
+      </c>
     </row>
     <row r="61" ht="13.65" customHeight="1">
       <c r="A61" t="s" s="45">
         <v>173</v>
       </c>
       <c r="B61" s="46"/>
-      <c r="C61" t="s" s="45">
-        <v>174</v>
-      </c>
+      <c r="C61" s="45"/>
       <c r="D61" s="6"/>
       <c r="E61" s="6"/>
       <c r="F61" s="6"/>
@@ -5799,15 +6062,16 @@
         <v>56</v>
       </c>
       <c r="N61" s="7"/>
+      <c r="O61" t="s" s="30">
+        <v>263</v>
+      </c>
     </row>
     <row r="62" ht="13.65" customHeight="1">
       <c r="A62" t="s" s="2">
         <v>175</v>
       </c>
       <c r="B62" s="6"/>
-      <c r="C62" t="s" s="2">
-        <v>174</v>
-      </c>
+      <c r="C62" s="2"/>
       <c r="D62" s="6"/>
       <c r="E62" s="6"/>
       <c r="F62" s="6"/>
@@ -5827,15 +6091,16 @@
         <v>56</v>
       </c>
       <c r="N62" s="7"/>
+      <c r="O62" t="s" s="30">
+        <v>263</v>
+      </c>
     </row>
     <row r="63" ht="13.65" customHeight="1">
       <c r="A63" t="s" s="2">
         <v>176</v>
       </c>
       <c r="B63" s="6"/>
-      <c r="C63" t="s" s="2">
-        <v>174</v>
-      </c>
+      <c r="C63" s="2"/>
       <c r="D63" s="6"/>
       <c r="E63" s="6"/>
       <c r="F63" s="6"/>
@@ -5855,15 +6120,16 @@
         <v>56</v>
       </c>
       <c r="N63" s="7"/>
+      <c r="O63" t="s" s="30">
+        <v>263</v>
+      </c>
     </row>
     <row r="64" ht="13.65" customHeight="1">
       <c r="A64" t="s" s="2">
         <v>177</v>
       </c>
       <c r="B64" s="6"/>
-      <c r="C64" t="s" s="2">
-        <v>174</v>
-      </c>
+      <c r="C64" s="2"/>
       <c r="D64" s="6"/>
       <c r="E64" s="6"/>
       <c r="F64" s="6"/>
@@ -5883,15 +6149,16 @@
         <v>56</v>
       </c>
       <c r="N64" s="7"/>
+      <c r="O64" t="s" s="30">
+        <v>263</v>
+      </c>
     </row>
     <row r="65" ht="13.65" customHeight="1">
       <c r="A65" t="s" s="2">
         <v>178</v>
       </c>
       <c r="B65" s="6"/>
-      <c r="C65" t="s" s="2">
-        <v>174</v>
-      </c>
+      <c r="C65" s="2"/>
       <c r="D65" s="6"/>
       <c r="E65" s="6"/>
       <c r="F65" s="6"/>
@@ -5911,15 +6178,16 @@
         <v>56</v>
       </c>
       <c r="N65" s="7"/>
+      <c r="O65" t="s" s="30">
+        <v>263</v>
+      </c>
     </row>
     <row r="66" ht="13.65" customHeight="1">
       <c r="A66" t="s" s="2">
         <v>179</v>
       </c>
       <c r="B66" s="6"/>
-      <c r="C66" t="s" s="2">
-        <v>174</v>
-      </c>
+      <c r="C66" s="2"/>
       <c r="D66" s="6"/>
       <c r="E66" s="6"/>
       <c r="F66" s="6"/>
@@ -5939,15 +6207,16 @@
         <v>56</v>
       </c>
       <c r="N66" s="7"/>
+      <c r="O66" t="s" s="30">
+        <v>263</v>
+      </c>
     </row>
     <row r="67" ht="13.65" customHeight="1">
       <c r="A67" t="s" s="2">
         <v>180</v>
       </c>
       <c r="B67" s="6"/>
-      <c r="C67" t="s" s="2">
-        <v>174</v>
-      </c>
+      <c r="C67" s="2"/>
       <c r="D67" s="6"/>
       <c r="E67" s="6"/>
       <c r="F67" s="6"/>
@@ -5967,15 +6236,16 @@
         <v>56</v>
       </c>
       <c r="N67" s="7"/>
+      <c r="O67" t="s" s="30">
+        <v>263</v>
+      </c>
     </row>
     <row r="68" ht="13.65" customHeight="1">
       <c r="A68" t="s" s="2">
         <v>181</v>
       </c>
       <c r="B68" s="6"/>
-      <c r="C68" t="s" s="2">
-        <v>174</v>
-      </c>
+      <c r="C68" s="2"/>
       <c r="D68" s="6"/>
       <c r="E68" s="6"/>
       <c r="F68" s="6"/>
@@ -5995,15 +6265,16 @@
         <v>56</v>
       </c>
       <c r="N68" s="7"/>
+      <c r="O68" t="s" s="30">
+        <v>263</v>
+      </c>
     </row>
     <row r="69" ht="13.65" customHeight="1">
       <c r="A69" t="s" s="2">
         <v>182</v>
       </c>
       <c r="B69" s="6"/>
-      <c r="C69" t="s" s="2">
-        <v>174</v>
-      </c>
+      <c r="C69" s="2"/>
       <c r="D69" s="6"/>
       <c r="E69" s="6"/>
       <c r="F69" s="6"/>
@@ -6023,15 +6294,16 @@
         <v>56</v>
       </c>
       <c r="N69" s="7"/>
+      <c r="O69" t="s" s="30">
+        <v>263</v>
+      </c>
     </row>
     <row r="70" ht="13.65" customHeight="1">
       <c r="A70" t="s" s="2">
         <v>183</v>
       </c>
       <c r="B70" s="6"/>
-      <c r="C70" t="s" s="2">
-        <v>174</v>
-      </c>
+      <c r="C70" s="2"/>
       <c r="D70" s="6"/>
       <c r="E70" s="6"/>
       <c r="F70" s="6"/>
@@ -6051,15 +6323,16 @@
         <v>56</v>
       </c>
       <c r="N70" s="7"/>
+      <c r="O70" t="s" s="30">
+        <v>263</v>
+      </c>
     </row>
     <row r="71" ht="13.65" customHeight="1">
       <c r="A71" t="s" s="2">
         <v>184</v>
       </c>
       <c r="B71" s="6"/>
-      <c r="C71" t="s" s="2">
-        <v>174</v>
-      </c>
+      <c r="C71" s="2"/>
       <c r="D71" s="6"/>
       <c r="E71" s="6"/>
       <c r="F71" s="6"/>
@@ -6079,15 +6352,16 @@
         <v>56</v>
       </c>
       <c r="N71" s="7"/>
+      <c r="O71" t="s" s="30">
+        <v>263</v>
+      </c>
     </row>
     <row r="72" ht="13.65" customHeight="1">
       <c r="A72" t="s" s="2">
         <v>185</v>
       </c>
       <c r="B72" s="6"/>
-      <c r="C72" t="s" s="2">
-        <v>174</v>
-      </c>
+      <c r="C72" s="2"/>
       <c r="D72" s="6"/>
       <c r="E72" s="6"/>
       <c r="F72" s="6"/>
@@ -6107,15 +6381,16 @@
         <v>56</v>
       </c>
       <c r="N72" s="7"/>
+      <c r="O72" t="s" s="30">
+        <v>263</v>
+      </c>
     </row>
     <row r="73" ht="13.65" customHeight="1">
       <c r="A73" t="s" s="2">
         <v>186</v>
       </c>
       <c r="B73" s="6"/>
-      <c r="C73" t="s" s="2">
-        <v>174</v>
-      </c>
+      <c r="C73" s="2"/>
       <c r="D73" s="6"/>
       <c r="E73" s="6"/>
       <c r="F73" s="6"/>
@@ -6135,15 +6410,16 @@
         <v>56</v>
       </c>
       <c r="N73" s="7"/>
+      <c r="O73" t="s" s="30">
+        <v>263</v>
+      </c>
     </row>
     <row r="74" ht="13.65" customHeight="1">
       <c r="A74" t="s" s="2">
         <v>187</v>
       </c>
       <c r="B74" s="6"/>
-      <c r="C74" t="s" s="2">
-        <v>188</v>
-      </c>
+      <c r="C74" s="2"/>
       <c r="D74" s="6"/>
       <c r="E74" s="6"/>
       <c r="F74" s="6"/>
@@ -6163,15 +6439,16 @@
         <v>56</v>
       </c>
       <c r="N74" s="7"/>
+      <c r="O74" t="s" s="30">
+        <v>264</v>
+      </c>
     </row>
     <row r="75" ht="13.65" customHeight="1">
       <c r="A75" t="s" s="2">
         <v>189</v>
       </c>
       <c r="B75" s="6"/>
-      <c r="C75" t="s" s="2">
-        <v>188</v>
-      </c>
+      <c r="C75" s="2"/>
       <c r="D75" s="6"/>
       <c r="E75" s="6"/>
       <c r="F75" s="6"/>
@@ -6191,15 +6468,16 @@
         <v>56</v>
       </c>
       <c r="N75" s="7"/>
+      <c r="O75" t="s" s="30">
+        <v>264</v>
+      </c>
     </row>
     <row r="76" ht="13.65" customHeight="1">
       <c r="A76" t="s" s="2">
         <v>190</v>
       </c>
       <c r="B76" s="6"/>
-      <c r="C76" t="s" s="2">
-        <v>188</v>
-      </c>
+      <c r="C76" s="2"/>
       <c r="D76" s="6"/>
       <c r="E76" s="6"/>
       <c r="F76" s="6"/>
@@ -6219,15 +6497,16 @@
         <v>56</v>
       </c>
       <c r="N76" s="7"/>
+      <c r="O76" t="s" s="30">
+        <v>264</v>
+      </c>
     </row>
     <row r="77" ht="13.65" customHeight="1">
       <c r="A77" t="s" s="2">
         <v>191</v>
       </c>
       <c r="B77" s="6"/>
-      <c r="C77" t="s" s="2">
-        <v>188</v>
-      </c>
+      <c r="C77" s="2"/>
       <c r="D77" s="6"/>
       <c r="E77" s="6"/>
       <c r="F77" s="6"/>
@@ -6247,15 +6526,16 @@
         <v>56</v>
       </c>
       <c r="N77" s="7"/>
+      <c r="O77" t="s" s="30">
+        <v>264</v>
+      </c>
     </row>
     <row r="78" ht="13.65" customHeight="1">
       <c r="A78" t="s" s="2">
         <v>192</v>
       </c>
       <c r="B78" s="6"/>
-      <c r="C78" t="s" s="2">
-        <v>188</v>
-      </c>
+      <c r="C78" s="2"/>
       <c r="D78" s="6"/>
       <c r="E78" s="6"/>
       <c r="F78" s="6"/>
@@ -6275,15 +6555,16 @@
         <v>56</v>
       </c>
       <c r="N78" s="7"/>
+      <c r="O78" t="s" s="30">
+        <v>264</v>
+      </c>
     </row>
     <row r="79" ht="13.65" customHeight="1">
       <c r="A79" t="s" s="2">
         <v>193</v>
       </c>
       <c r="B79" s="6"/>
-      <c r="C79" t="s" s="2">
-        <v>188</v>
-      </c>
+      <c r="C79" s="2"/>
       <c r="D79" s="6"/>
       <c r="E79" s="6"/>
       <c r="F79" s="6"/>
@@ -6303,15 +6584,16 @@
         <v>56</v>
       </c>
       <c r="N79" s="7"/>
+      <c r="O79" t="s" s="30">
+        <v>264</v>
+      </c>
     </row>
     <row r="80" ht="13.65" customHeight="1">
       <c r="A80" t="s" s="2">
         <v>194</v>
       </c>
       <c r="B80" s="6"/>
-      <c r="C80" t="s" s="2">
-        <v>188</v>
-      </c>
+      <c r="C80" s="2"/>
       <c r="D80" s="6"/>
       <c r="E80" s="6"/>
       <c r="F80" s="6"/>
@@ -6331,6 +6613,9 @@
         <v>56</v>
       </c>
       <c r="N80" s="7"/>
+      <c r="O80" t="s" s="30">
+        <v>264</v>
+      </c>
     </row>
     <row r="81" ht="13.65" customHeight="1">
       <c r="A81" s="2"/>
@@ -21212,15 +21497,15 @@
   <dimension ref="A1:H946"/>
   <sheetFormatPr defaultColWidth="12.6667" defaultRowHeight="15.75" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="19.6719" style="47" customWidth="1"/>
-    <col min="2" max="2" width="50.8516" style="47" customWidth="1"/>
-    <col min="3" max="3" width="45.8516" style="47" customWidth="1"/>
-    <col min="4" max="4" width="48.5" style="47" customWidth="1"/>
-    <col min="5" max="5" width="21" style="47" customWidth="1"/>
-    <col min="6" max="6" width="23" style="47" customWidth="1"/>
-    <col min="7" max="7" width="26.3516" style="47" customWidth="1"/>
-    <col min="8" max="8" width="26.5" style="47" customWidth="1"/>
-    <col min="9" max="16384" width="12.6719" style="47" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" style="47" width="19.6719"/>
+    <col min="2" max="2" customWidth="true" style="47" width="50.8516"/>
+    <col min="3" max="3" customWidth="true" style="47" width="45.8516"/>
+    <col min="4" max="4" customWidth="true" style="47" width="48.5"/>
+    <col min="5" max="5" customWidth="true" style="47" width="21.0"/>
+    <col min="6" max="6" customWidth="true" style="47" width="23.0"/>
+    <col min="7" max="7" customWidth="true" style="47" width="26.3516"/>
+    <col min="8" max="8" customWidth="true" style="47" width="26.5"/>
+    <col min="9" max="16384" customWidth="true" style="47" width="12.6719"/>
   </cols>
   <sheetData>
     <row r="1" ht="13.65" customHeight="1">
@@ -30774,8 +31059,8 @@
   <dimension ref="A1:E73"/>
   <sheetFormatPr defaultColWidth="16.3333" defaultRowHeight="13.45" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="5" width="16.3516" style="52" customWidth="1"/>
-    <col min="6" max="16384" width="16.3516" style="52" customWidth="1"/>
+    <col min="1" max="5" customWidth="true" style="52" width="16.3516"/>
+    <col min="6" max="16384" customWidth="true" style="52" width="16.3516"/>
   </cols>
   <sheetData>
     <row r="1" ht="13.2" customHeight="1">
@@ -31591,15 +31876,15 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr defaultColWidth="16.3333" defaultRowHeight="13.45" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="19.6719" style="64" customWidth="1"/>
-    <col min="2" max="2" width="38" style="64" customWidth="1"/>
-    <col min="3" max="3" width="12.5" style="64" customWidth="1"/>
-    <col min="4" max="4" width="19.8516" style="64" customWidth="1"/>
-    <col min="5" max="6" width="16.3516" style="64" customWidth="1"/>
-    <col min="7" max="16384" width="16.3516" style="64" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" style="64" width="19.6719"/>
+    <col min="2" max="2" customWidth="true" style="64" width="38.0"/>
+    <col min="3" max="3" customWidth="true" style="64" width="12.5"/>
+    <col min="4" max="4" customWidth="true" style="64" width="19.8516"/>
+    <col min="5" max="6" customWidth="true" style="64" width="16.3516"/>
+    <col min="7" max="16384" customWidth="true" style="64" width="16.3516"/>
   </cols>
   <sheetData>
     <row r="1" ht="13.2" customHeight="1">
@@ -31621,14 +31906,15 @@
       <c r="F1" t="s" s="11">
         <v>219</v>
       </c>
+      <c r="G1" t="s" s="64">
+        <v>282</v>
+      </c>
     </row>
     <row r="2" ht="13.2" customHeight="1">
       <c r="A2" t="s" s="68">
         <v>49</v>
       </c>
-      <c r="B2" t="s" s="69">
-        <v>220</v>
-      </c>
+      <c r="B2" s="69"/>
       <c r="C2" t="s" s="69">
         <v>57</v>
       </c>
@@ -31640,15 +31926,16 @@
       </c>
       <c r="F2" t="s" s="71">
         <v>221</v>
+      </c>
+      <c r="G2" t="s" s="64">
+        <v>283</v>
       </c>
     </row>
     <row r="3" ht="13" customHeight="1">
       <c r="A3" t="s" s="68">
         <v>49</v>
       </c>
-      <c r="B3" t="s" s="69">
-        <v>220</v>
-      </c>
+      <c r="B3" s="69"/>
       <c r="C3" t="s" s="69">
         <v>59</v>
       </c>
@@ -31660,15 +31947,16 @@
       </c>
       <c r="F3" t="s" s="73">
         <v>221</v>
+      </c>
+      <c r="G3" t="s" s="64">
+        <v>283</v>
       </c>
     </row>
     <row r="4" ht="13" customHeight="1">
       <c r="A4" t="s" s="68">
         <v>49</v>
       </c>
-      <c r="B4" t="s" s="69">
-        <v>220</v>
-      </c>
+      <c r="B4" s="69"/>
       <c r="C4" t="s" s="69">
         <v>61</v>
       </c>
@@ -31680,15 +31968,16 @@
       </c>
       <c r="F4" t="s" s="73">
         <v>221</v>
+      </c>
+      <c r="G4" t="s" s="64">
+        <v>283</v>
       </c>
     </row>
     <row r="5" ht="13" customHeight="1">
       <c r="A5" t="s" s="68">
         <v>49</v>
       </c>
-      <c r="B5" t="s" s="69">
-        <v>220</v>
-      </c>
+      <c r="B5" s="69"/>
       <c r="C5" t="s" s="69">
         <v>93</v>
       </c>
@@ -31700,15 +31989,16 @@
       </c>
       <c r="F5" t="s" s="73">
         <v>221</v>
+      </c>
+      <c r="G5" t="s" s="64">
+        <v>283</v>
       </c>
     </row>
     <row r="6" ht="13" customHeight="1">
       <c r="A6" t="s" s="68">
         <v>49</v>
       </c>
-      <c r="B6" t="s" s="69">
-        <v>220</v>
-      </c>
+      <c r="B6" s="69"/>
       <c r="C6" t="s" s="69">
         <v>102</v>
       </c>
@@ -31720,15 +32010,16 @@
       </c>
       <c r="F6" t="s" s="73">
         <v>221</v>
+      </c>
+      <c r="G6" t="s" s="64">
+        <v>283</v>
       </c>
     </row>
     <row r="7" ht="13" customHeight="1">
       <c r="A7" t="s" s="68">
         <v>49</v>
       </c>
-      <c r="B7" t="s" s="69">
-        <v>220</v>
-      </c>
+      <c r="B7" s="69"/>
       <c r="C7" t="s" s="69">
         <v>158</v>
       </c>
@@ -31740,15 +32031,16 @@
       </c>
       <c r="F7" t="s" s="73">
         <v>221</v>
+      </c>
+      <c r="G7" t="s" s="64">
+        <v>283</v>
       </c>
     </row>
     <row r="8" ht="13" customHeight="1">
       <c r="A8" t="s" s="68">
         <v>49</v>
       </c>
-      <c r="B8" t="s" s="69">
-        <v>220</v>
-      </c>
+      <c r="B8" s="69"/>
       <c r="C8" t="s" s="69">
         <v>95</v>
       </c>
@@ -31760,15 +32052,16 @@
       </c>
       <c r="F8" t="s" s="73">
         <v>221</v>
+      </c>
+      <c r="G8" t="s" s="64">
+        <v>283</v>
       </c>
     </row>
     <row r="9" ht="13" customHeight="1">
       <c r="A9" t="s" s="68">
         <v>49</v>
       </c>
-      <c r="B9" t="s" s="69">
-        <v>220</v>
-      </c>
+      <c r="B9" s="69"/>
       <c r="C9" t="s" s="69">
         <v>109</v>
       </c>
@@ -31780,15 +32073,16 @@
       </c>
       <c r="F9" t="s" s="73">
         <v>221</v>
+      </c>
+      <c r="G9" t="s" s="64">
+        <v>283</v>
       </c>
     </row>
     <row r="10" ht="13" customHeight="1">
       <c r="A10" t="s" s="68">
         <v>49</v>
       </c>
-      <c r="B10" t="s" s="69">
-        <v>220</v>
-      </c>
+      <c r="B10" s="69"/>
       <c r="C10" t="s" s="69">
         <v>111</v>
       </c>
@@ -31800,15 +32094,16 @@
       </c>
       <c r="F10" t="s" s="73">
         <v>221</v>
+      </c>
+      <c r="G10" t="s" s="64">
+        <v>283</v>
       </c>
     </row>
     <row r="11" ht="13" customHeight="1">
       <c r="A11" t="s" s="68">
         <v>117</v>
       </c>
-      <c r="B11" t="s" s="69">
-        <v>223</v>
-      </c>
+      <c r="B11" s="69"/>
       <c r="C11" t="s" s="69">
         <v>49</v>
       </c>
@@ -31820,15 +32115,16 @@
       </c>
       <c r="F11" t="s" s="73">
         <v>221</v>
+      </c>
+      <c r="G11" t="s" s="64">
+        <v>284</v>
       </c>
     </row>
     <row r="12" ht="13" customHeight="1">
       <c r="A12" t="s" s="68">
         <v>49</v>
       </c>
-      <c r="B12" t="s" s="69">
-        <v>220</v>
-      </c>
+      <c r="B12" s="69"/>
       <c r="C12" t="s" s="69">
         <v>121</v>
       </c>
@@ -31840,15 +32136,16 @@
       </c>
       <c r="F12" t="s" s="73">
         <v>221</v>
+      </c>
+      <c r="G12" t="s" s="64">
+        <v>283</v>
       </c>
     </row>
     <row r="13" ht="13" customHeight="1">
       <c r="A13" t="s" s="68">
         <v>49</v>
       </c>
-      <c r="B13" t="s" s="69">
-        <v>220</v>
-      </c>
+      <c r="B13" s="69"/>
       <c r="C13" t="s" s="69">
         <v>138</v>
       </c>
@@ -31860,15 +32157,16 @@
       </c>
       <c r="F13" t="s" s="73">
         <v>221</v>
+      </c>
+      <c r="G13" t="s" s="64">
+        <v>283</v>
       </c>
     </row>
     <row r="14" ht="13" customHeight="1">
       <c r="A14" t="s" s="68">
         <v>82</v>
       </c>
-      <c r="B14" t="s" s="69">
-        <v>223</v>
-      </c>
+      <c r="B14" s="69"/>
       <c r="C14" t="s" s="69">
         <v>57</v>
       </c>
@@ -31880,15 +32178,16 @@
       </c>
       <c r="F14" t="s" s="73">
         <v>221</v>
+      </c>
+      <c r="G14" t="s" s="64">
+        <v>284</v>
       </c>
     </row>
     <row r="15" ht="13" customHeight="1">
       <c r="A15" t="s" s="68">
         <v>49</v>
       </c>
-      <c r="B15" t="s" s="69">
-        <v>223</v>
-      </c>
+      <c r="B15" s="69"/>
       <c r="C15" t="s" s="69">
         <v>57</v>
       </c>
@@ -31900,15 +32199,16 @@
       </c>
       <c r="F15" t="s" s="73">
         <v>221</v>
+      </c>
+      <c r="G15" t="s" s="64">
+        <v>284</v>
       </c>
     </row>
     <row r="16" ht="13" customHeight="1">
       <c r="A16" t="s" s="68">
         <v>59</v>
       </c>
-      <c r="B16" t="s" s="69">
-        <v>223</v>
-      </c>
+      <c r="B16" s="69"/>
       <c r="C16" t="s" s="69">
         <v>57</v>
       </c>
@@ -31920,15 +32220,16 @@
       </c>
       <c r="F16" t="s" s="73">
         <v>221</v>
+      </c>
+      <c r="G16" t="s" s="64">
+        <v>284</v>
       </c>
     </row>
     <row r="17" ht="13" customHeight="1">
       <c r="A17" t="s" s="68">
         <v>61</v>
       </c>
-      <c r="B17" t="s" s="69">
-        <v>223</v>
-      </c>
+      <c r="B17" s="69"/>
       <c r="C17" t="s" s="69">
         <v>57</v>
       </c>
@@ -31940,15 +32241,16 @@
       </c>
       <c r="F17" t="s" s="73">
         <v>221</v>
+      </c>
+      <c r="G17" t="s" s="64">
+        <v>284</v>
       </c>
     </row>
     <row r="18" ht="13" customHeight="1">
       <c r="A18" t="s" s="68">
         <v>84</v>
       </c>
-      <c r="B18" t="s" s="69">
-        <v>223</v>
-      </c>
+      <c r="B18" s="69"/>
       <c r="C18" t="s" s="69">
         <v>57</v>
       </c>
@@ -31960,15 +32262,16 @@
       </c>
       <c r="F18" t="s" s="73">
         <v>221</v>
+      </c>
+      <c r="G18" t="s" s="64">
+        <v>284</v>
       </c>
     </row>
     <row r="19" ht="13" customHeight="1">
       <c r="A19" t="s" s="68">
         <v>93</v>
       </c>
-      <c r="B19" t="s" s="69">
-        <v>223</v>
-      </c>
+      <c r="B19" s="69"/>
       <c r="C19" t="s" s="69">
         <v>57</v>
       </c>
@@ -31980,15 +32283,16 @@
       </c>
       <c r="F19" t="s" s="73">
         <v>221</v>
+      </c>
+      <c r="G19" t="s" s="64">
+        <v>284</v>
       </c>
     </row>
     <row r="20" ht="13" customHeight="1">
       <c r="A20" t="s" s="68">
         <v>97</v>
       </c>
-      <c r="B20" t="s" s="69">
-        <v>223</v>
-      </c>
+      <c r="B20" s="69"/>
       <c r="C20" t="s" s="69">
         <v>57</v>
       </c>
@@ -32000,15 +32304,16 @@
       </c>
       <c r="F20" t="s" s="73">
         <v>221</v>
+      </c>
+      <c r="G20" t="s" s="64">
+        <v>284</v>
       </c>
     </row>
     <row r="21" ht="13" customHeight="1">
       <c r="A21" t="s" s="74">
         <v>57</v>
       </c>
-      <c r="B21" t="s" s="75">
-        <v>220</v>
-      </c>
+      <c r="B21" s="75"/>
       <c r="C21" t="s" s="75">
         <v>150</v>
       </c>
@@ -32020,6 +32325,9 @@
       </c>
       <c r="F21" t="s" s="77">
         <v>221</v>
+      </c>
+      <c r="G21" t="s" s="64">
+        <v>283</v>
       </c>
     </row>
   </sheetData>
@@ -32039,10 +32347,10 @@
   <dimension ref="A1:I10"/>
   <sheetFormatPr defaultColWidth="16.3333" defaultRowHeight="13.45" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="3" width="16.3516" style="78" customWidth="1"/>
-    <col min="4" max="4" width="43" style="78" customWidth="1"/>
-    <col min="5" max="9" width="16.3516" style="78" customWidth="1"/>
-    <col min="10" max="16384" width="16.3516" style="78" customWidth="1"/>
+    <col min="1" max="3" customWidth="true" style="78" width="16.3516"/>
+    <col min="4" max="4" customWidth="true" style="78" width="43.0"/>
+    <col min="5" max="9" customWidth="true" style="78" width="16.3516"/>
+    <col min="10" max="16384" customWidth="true" style="78" width="16.3516"/>
   </cols>
   <sheetData>
     <row r="1" ht="13.45" customHeight="1">

</xml_diff>